<commit_message>
Fix template generation script to populate Excel file correctly
</commit_message>
<xml_diff>
--- a/Populated_Parity_Template.xlsx
+++ b/Populated_Parity_Template.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="277">
   <si>
     <t>project_name</t>
   </si>
@@ -125,6 +125,150 @@
     <t>rera_registration_no</t>
   </si>
   <si>
+    <t>Rainbow Mayfair</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>Hullahalli, Bengaluru</t>
+  </si>
+  <si>
+    <t>4 Acre</t>
+  </si>
+  <si>
+    <t>Lake-Facing Serenity</t>
+  </si>
+  <si>
+    <t>UnderConstruction</t>
+  </si>
+  <si>
+    <t>Villas</t>
+  </si>
+  <si>
+    <t>PRM/KA/RERA/1251/308/PR/190325/007593</t>
+  </si>
+  <si>
+    <t>SOBHA Neopolis</t>
+  </si>
+  <si>
+    <t>Panathur Main Road, ORR IT Corridor</t>
+  </si>
+  <si>
+    <t>25 Acres</t>
+  </si>
+  <si>
+    <t>Greek / Santorini Theme</t>
+  </si>
+  <si>
+    <t>Premium Residential Township</t>
+  </si>
+  <si>
+    <t>PRM/KA/RERA/1251/446/PR/200923/006269</t>
+  </si>
+  <si>
+    <t>Godrej Woods</t>
+  </si>
+  <si>
+    <t>Thanisandra Main Road</t>
+  </si>
+  <si>
+    <t>7 Acres</t>
+  </si>
+  <si>
+    <t>Forest-Themed</t>
+  </si>
+  <si>
+    <t>High-Rise Residential Apartments</t>
+  </si>
+  <si>
+    <t>PRM/KA/RERA/1251/472/PR/121125/008248</t>
+  </si>
+  <si>
+    <t>Brigade Belvedere</t>
+  </si>
+  <si>
+    <t>Budigere Cross</t>
+  </si>
+  <si>
+    <t>10.75 Acres</t>
+  </si>
+  <si>
+    <t>Premium High-Rise Urban Living</t>
+  </si>
+  <si>
+    <t>Residential Apartments</t>
+  </si>
+  <si>
+    <t>PRM/KA/RERA/1251/446/PR/240326/008549</t>
+  </si>
+  <si>
+    <t>Bren Aspera</t>
+  </si>
+  <si>
+    <t>Old Madras Road Corridor</t>
+  </si>
+  <si>
+    <t>4.39 Acres</t>
+  </si>
+  <si>
+    <t>Premium Community Living</t>
+  </si>
+  <si>
+    <t>Premium Residential Apartments</t>
+  </si>
+  <si>
+    <t>PRM/KA/RERA/1251/310/PR/300622/005028</t>
+  </si>
+  <si>
+    <t>Godrej Parkshire</t>
+  </si>
+  <si>
+    <t>Hoskote</t>
+  </si>
+  <si>
+    <t>13.8 Acres</t>
+  </si>
+  <si>
+    <t>Nature-Themed High-Rise Living</t>
+  </si>
+  <si>
+    <t>PRM/KA/RERA/1250/304/PR/090126/008393</t>
+  </si>
+  <si>
+    <t>Sattva Songbird</t>
+  </si>
+  <si>
+    <t>300 meters from Old Madras Road</t>
+  </si>
+  <si>
+    <t>16 Acres</t>
+  </si>
+  <si>
+    <t>Nature-Themed Township Living</t>
+  </si>
+  <si>
+    <t>Integrated Township</t>
+  </si>
+  <si>
+    <t>PRM/KA/RERA/1251/310/PR/270326/008557</t>
+  </si>
+  <si>
+    <t>SOBHA OneWorld</t>
+  </si>
+  <si>
+    <t>Old Madras Road</t>
+  </si>
+  <si>
+    <t>48 Acres</t>
+  </si>
+  <si>
+    <t>Next-generation integrated township</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
     <t>name</t>
   </si>
   <si>
@@ -155,6 +299,27 @@
     <t>financial_strength</t>
   </si>
   <si>
+    <t>Rainbow Properties</t>
+  </si>
+  <si>
+    <t>SOBHA Limited</t>
+  </si>
+  <si>
+    <t>Godrej Properties Limited</t>
+  </si>
+  <si>
+    <t>Brigade Group</t>
+  </si>
+  <si>
+    <t>Bren Corporation Pvt. Ltd.</t>
+  </si>
+  <si>
+    <t>Godrej Properties Ltd.</t>
+  </si>
+  <si>
+    <t>Sattva Group</t>
+  </si>
+  <si>
     <t>pros</t>
   </si>
   <si>
@@ -185,6 +350,99 @@
     <t>overall_rating</t>
   </si>
   <si>
+    <t>["Lakefront living","Vehicle-Free Zone","Large UDS"]</t>
+  </si>
+  <si>
+    <t>["Common wall structure","Far from metro"]</t>
+  </si>
+  <si>
+    <t>Lakefront living</t>
+  </si>
+  <si>
+    <t>IT professionals, families</t>
+  </si>
+  <si>
+    <t>["Theme: Greek Santorini","3 Clubhouses","Low Density"]</t>
+  </si>
+  <si>
+    <t>["High pricing","Traffic on Panathur road"]</t>
+  </si>
+  <si>
+    <t>Theme: Greek Santorini</t>
+  </si>
+  <si>
+    <t>IT Professionals (VP/Director level)</t>
+  </si>
+  <si>
+    <t>["Forest Living","Main Road Location"]</t>
+  </si>
+  <si>
+    <t>["Small 2BHK size"]</t>
+  </si>
+  <si>
+    <t>Forest Living</t>
+  </si>
+  <si>
+    <t>IT families</t>
+  </si>
+  <si>
+    <t>["High Rise 43 floors","Large units","Prime location"]</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>High Rise 43 floors</t>
+  </si>
+  <si>
+    <t>IT professionals, investors</t>
+  </si>
+  <si>
+    <t>["Low density","Established builder"]</t>
+  </si>
+  <si>
+    <t>["Only 3BHK available"]</t>
+  </si>
+  <si>
+    <t>Low density</t>
+  </si>
+  <si>
+    <t>IT Professionals + Investors</t>
+  </si>
+  <si>
+    <t>["Nature-Themed Township Living","Godrej brand","Large land parcel"]</t>
+  </si>
+  <si>
+    <t>["Hoskote distance"]</t>
+  </si>
+  <si>
+    <t>Investors, IT professionals</t>
+  </si>
+  <si>
+    <t>["16 Acres Township","Sattva Brand","STRR Growth"]</t>
+  </si>
+  <si>
+    <t>["Long Timeline"]</t>
+  </si>
+  <si>
+    <t>16 Acres Township</t>
+  </si>
+  <si>
+    <t>Investors + End Users</t>
+  </si>
+  <si>
+    <t>["SOBHA brand","48-acre township","Multiple unit options"]</t>
+  </si>
+  <si>
+    <t>["Possession details not shared"]</t>
+  </si>
+  <si>
+    <t>SOBHA brand</t>
+  </si>
+  <si>
+    <t>Investors, East Bengaluru buyers</t>
+  </si>
+  <si>
     <t>unitnumber</t>
   </si>
   <si>
@@ -227,6 +485,108 @@
     <t>status</t>
   </si>
   <si>
+    <t>U-1</t>
+  </si>
+  <si>
+    <t>4BHK</t>
+  </si>
+  <si>
+    <t>Available</t>
+  </si>
+  <si>
+    <t>U-2</t>
+  </si>
+  <si>
+    <t>U-3</t>
+  </si>
+  <si>
+    <t>U-4</t>
+  </si>
+  <si>
+    <t>5BHK</t>
+  </si>
+  <si>
+    <t>U-5</t>
+  </si>
+  <si>
+    <t>1 BHK</t>
+  </si>
+  <si>
+    <t>U-6</t>
+  </si>
+  <si>
+    <t>3 BHK</t>
+  </si>
+  <si>
+    <t>U-7</t>
+  </si>
+  <si>
+    <t>4 BHK</t>
+  </si>
+  <si>
+    <t>U-8</t>
+  </si>
+  <si>
+    <t>2 BHK</t>
+  </si>
+  <si>
+    <t>U-9</t>
+  </si>
+  <si>
+    <t>3 BHK Premium</t>
+  </si>
+  <si>
+    <t>U-10</t>
+  </si>
+  <si>
+    <t>3 BHK Luxe</t>
+  </si>
+  <si>
+    <t>U-11</t>
+  </si>
+  <si>
+    <t>U-12</t>
+  </si>
+  <si>
+    <t>U-13</t>
+  </si>
+  <si>
+    <t>U-14</t>
+  </si>
+  <si>
+    <t>U-15</t>
+  </si>
+  <si>
+    <t>U-16</t>
+  </si>
+  <si>
+    <t>U-17</t>
+  </si>
+  <si>
+    <t>U-18</t>
+  </si>
+  <si>
+    <t>U-19</t>
+  </si>
+  <si>
+    <t>U-20</t>
+  </si>
+  <si>
+    <t>Row House</t>
+  </si>
+  <si>
+    <t>U-21</t>
+  </si>
+  <si>
+    <t>U-22</t>
+  </si>
+  <si>
+    <t>U-23</t>
+  </si>
+  <si>
+    <t>U-24</t>
+  </si>
+  <si>
     <t>no_of_towers</t>
   </si>
   <si>
@@ -311,12 +671,66 @@
     <t>open_space_pct</t>
   </si>
   <si>
+    <t>Seismic-II zone compliant RCC framed structure</t>
+  </si>
+  <si>
+    <t>RCC-framed high-rise structure</t>
+  </si>
+  <si>
+    <t>RCC Framed Structure</t>
+  </si>
+  <si>
+    <t>RCC High-rise</t>
+  </si>
+  <si>
+    <t>RCC (Aluminium Formwork)</t>
+  </si>
+  <si>
+    <t>RCC High-Rise Structure</t>
+  </si>
+  <si>
+    <t>RCC / Shear Wall Structure</t>
+  </si>
+  <si>
+    <t>High-rise residential township</t>
+  </si>
+  <si>
     <t>category</t>
   </si>
   <si>
     <t>size_specs</t>
   </si>
   <si>
+    <t>Clubhouse</t>
+  </si>
+  <si>
+    <t>Main Clubhouse</t>
+  </si>
+  <si>
+    <t>11,000 Sq.ft</t>
+  </si>
+  <si>
+    <t>77,850 sq ft</t>
+  </si>
+  <si>
+    <t>20,000 Sq. Ft.</t>
+  </si>
+  <si>
+    <t>25,000 Sq.ft</t>
+  </si>
+  <si>
+    <t>15,000 Sq.ft</t>
+  </si>
+  <si>
+    <t>32,500 sq.ft</t>
+  </si>
+  <si>
+    <t>100,000 sqft</t>
+  </si>
+  <si>
+    <t>50,000 sqft</t>
+  </si>
+  <si>
     <t>distance_km</t>
   </si>
   <si>
@@ -348,6 +762,57 @@
   </si>
   <si>
     <t>busstopdistance</t>
+  </si>
+  <si>
+    <t>1 Kms</t>
+  </si>
+  <si>
+    <t>45-60 km</t>
+  </si>
+  <si>
+    <t>Heelalige</t>
+  </si>
+  <si>
+    <t>Upcoming Namma Metro Yellow Line</t>
+  </si>
+  <si>
+    <t>Immediate access</t>
+  </si>
+  <si>
+    <t>Metro Phase 2A/2B</t>
+  </si>
+  <si>
+    <t>0 km</t>
+  </si>
+  <si>
+    <t>25 mins</t>
+  </si>
+  <si>
+    <t>Yelahanka Junction</t>
+  </si>
+  <si>
+    <t>Upcoming Nagawara</t>
+  </si>
+  <si>
+    <t>25-30 km</t>
+  </si>
+  <si>
+    <t>KR Puram</t>
+  </si>
+  <si>
+    <t>KR Puram Metro</t>
+  </si>
+  <si>
+    <t>27-32 km</t>
+  </si>
+  <si>
+    <t>30-35 km</t>
+  </si>
+  <si>
+    <t>Whitefield</t>
+  </si>
+  <si>
+    <t>Whitefield Metro</t>
   </si>
   <si>
     <t>customer_name</t>
@@ -766,7 +1231,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AG1"/>
+  <dimension ref="A1:AG9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -868,6 +1333,310 @@
       </c>
       <c r="AG1" t="s">
         <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+      <c r="J2" t="s">
+        <v>37</v>
+      </c>
+      <c r="K2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S2" t="s">
+        <v>39</v>
+      </c>
+      <c r="U2">
+        <v>64</v>
+      </c>
+      <c r="W2">
+        <v>10200000</v>
+      </c>
+      <c r="X2">
+        <v>30600000</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I3">
+        <v>5</v>
+      </c>
+      <c r="J3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K3" t="s">
+        <v>38</v>
+      </c>
+      <c r="S3" t="s">
+        <v>45</v>
+      </c>
+      <c r="U3">
+        <v>1875</v>
+      </c>
+      <c r="W3">
+        <v>12000000</v>
+      </c>
+      <c r="X3">
+        <v>36000000</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4" t="s">
+        <v>50</v>
+      </c>
+      <c r="K4" t="s">
+        <v>38</v>
+      </c>
+      <c r="S4" t="s">
+        <v>51</v>
+      </c>
+      <c r="U4">
+        <v>558</v>
+      </c>
+      <c r="W4">
+        <v>12000000</v>
+      </c>
+      <c r="X4">
+        <v>36000000</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" t="s">
+        <v>54</v>
+      </c>
+      <c r="H5" t="s">
+        <v>55</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5" t="s">
+        <v>56</v>
+      </c>
+      <c r="K5" t="s">
+        <v>38</v>
+      </c>
+      <c r="S5" t="s">
+        <v>57</v>
+      </c>
+      <c r="U5">
+        <v>1750</v>
+      </c>
+      <c r="W5">
+        <v>11761000</v>
+      </c>
+      <c r="X5">
+        <v>35283000</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" t="s">
+        <v>60</v>
+      </c>
+      <c r="H6" t="s">
+        <v>61</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6" t="s">
+        <v>62</v>
+      </c>
+      <c r="K6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S6" t="s">
+        <v>63</v>
+      </c>
+      <c r="U6">
+        <v>394</v>
+      </c>
+      <c r="W6">
+        <v>9800000</v>
+      </c>
+      <c r="X6">
+        <v>29400000</v>
+      </c>
+      <c r="AG6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" t="s">
+        <v>66</v>
+      </c>
+      <c r="H7" t="s">
+        <v>67</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="J7" t="s">
+        <v>68</v>
+      </c>
+      <c r="K7" t="s">
+        <v>38</v>
+      </c>
+      <c r="S7" t="s">
+        <v>63</v>
+      </c>
+      <c r="U7">
+        <v>1100</v>
+      </c>
+      <c r="W7">
+        <v>12300000</v>
+      </c>
+      <c r="X7">
+        <v>36900000</v>
+      </c>
+      <c r="AG7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>71</v>
+      </c>
+      <c r="H8" t="s">
+        <v>72</v>
+      </c>
+      <c r="I8">
+        <v>2</v>
+      </c>
+      <c r="J8" t="s">
+        <v>73</v>
+      </c>
+      <c r="K8" t="s">
+        <v>38</v>
+      </c>
+      <c r="S8" t="s">
+        <v>74</v>
+      </c>
+      <c r="U8">
+        <v>1679</v>
+      </c>
+      <c r="W8">
+        <v>10500000</v>
+      </c>
+      <c r="X8">
+        <v>31500000</v>
+      </c>
+      <c r="AG8" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" t="s">
+        <v>77</v>
+      </c>
+      <c r="H9" t="s">
+        <v>78</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9" t="s">
+        <v>79</v>
+      </c>
+      <c r="K9" t="s">
+        <v>38</v>
+      </c>
+      <c r="S9" t="s">
+        <v>74</v>
+      </c>
+      <c r="U9">
+        <v>3484</v>
+      </c>
+      <c r="W9">
+        <v>11500000</v>
+      </c>
+      <c r="X9">
+        <v>34500000</v>
+      </c>
+      <c r="AG9" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -878,7 +1647,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -886,19 +1655,155 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>103</v>
+        <v>241</v>
       </c>
       <c r="C1" t="s">
-        <v>104</v>
+        <v>242</v>
       </c>
       <c r="D1" t="s">
-        <v>105</v>
+        <v>243</v>
       </c>
       <c r="E1" t="s">
-        <v>106</v>
+        <v>244</v>
       </c>
       <c r="F1" t="s">
-        <v>107</v>
+        <v>245</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>246</v>
+      </c>
+      <c r="C2" t="s">
+        <v>247</v>
+      </c>
+      <c r="D2" t="s">
+        <v>248</v>
+      </c>
+      <c r="E2" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" t="s">
+        <v>250</v>
+      </c>
+      <c r="C3" t="s">
+        <v>247</v>
+      </c>
+      <c r="D3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E3" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" t="s">
+        <v>252</v>
+      </c>
+      <c r="C4" t="s">
+        <v>253</v>
+      </c>
+      <c r="D4" t="s">
+        <v>254</v>
+      </c>
+      <c r="E4" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C5" t="s">
+        <v>256</v>
+      </c>
+      <c r="D5" t="s">
+        <v>257</v>
+      </c>
+      <c r="E5" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6" t="s">
+        <v>252</v>
+      </c>
+      <c r="C6" t="s">
+        <v>259</v>
+      </c>
+      <c r="D6" t="s">
+        <v>257</v>
+      </c>
+      <c r="E6" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" t="s">
+        <v>252</v>
+      </c>
+      <c r="C7" t="s">
+        <v>260</v>
+      </c>
+      <c r="D7" t="s">
+        <v>261</v>
+      </c>
+      <c r="E7" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" t="s">
+        <v>252</v>
+      </c>
+      <c r="C8" t="s">
+        <v>256</v>
+      </c>
+      <c r="D8" t="s">
+        <v>257</v>
+      </c>
+      <c r="E8" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" t="s">
+        <v>252</v>
+      </c>
+      <c r="C9" t="s">
+        <v>260</v>
+      </c>
+      <c r="D9" t="s">
+        <v>257</v>
+      </c>
+      <c r="E9" t="s">
+        <v>262</v>
       </c>
     </row>
   </sheetData>
@@ -917,22 +1822,22 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>108</v>
+        <v>263</v>
       </c>
       <c r="C1" t="s">
-        <v>109</v>
+        <v>264</v>
       </c>
       <c r="D1" t="s">
-        <v>110</v>
+        <v>265</v>
       </c>
       <c r="E1" t="s">
-        <v>111</v>
+        <v>266</v>
       </c>
       <c r="F1" t="s">
-        <v>66</v>
+        <v>152</v>
       </c>
       <c r="G1" t="s">
-        <v>112</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -951,19 +1856,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>81</v>
       </c>
       <c r="C1" t="s">
-        <v>113</v>
+        <v>268</v>
       </c>
       <c r="D1" t="s">
-        <v>114</v>
+        <v>269</v>
       </c>
       <c r="E1" t="s">
-        <v>66</v>
+        <v>152</v>
       </c>
       <c r="F1" t="s">
-        <v>115</v>
+        <v>270</v>
       </c>
     </row>
   </sheetData>
@@ -979,16 +1884,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>113</v>
+        <v>268</v>
       </c>
       <c r="B1" t="s">
-        <v>116</v>
+        <v>271</v>
       </c>
       <c r="C1" t="s">
-        <v>117</v>
+        <v>272</v>
       </c>
       <c r="D1" t="s">
-        <v>118</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>
@@ -1004,16 +1909,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>119</v>
+        <v>274</v>
       </c>
       <c r="B1" t="s">
-        <v>120</v>
+        <v>275</v>
       </c>
       <c r="C1" t="s">
-        <v>66</v>
+        <v>152</v>
       </c>
       <c r="D1" t="s">
-        <v>121</v>
+        <v>276</v>
       </c>
     </row>
   </sheetData>
@@ -1024,7 +1929,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -1032,34 +1937,98 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E1" t="s">
+        <v>84</v>
+      </c>
+      <c r="F1" t="s">
+        <v>85</v>
+      </c>
+      <c r="G1" t="s">
+        <v>86</v>
+      </c>
+      <c r="H1" t="s">
+        <v>87</v>
+      </c>
+      <c r="I1" t="s">
+        <v>88</v>
+      </c>
+      <c r="J1" t="s">
+        <v>89</v>
+      </c>
+      <c r="K1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E1" t="s">
-        <v>36</v>
-      </c>
-      <c r="F1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G1" t="s">
-        <v>38</v>
-      </c>
-      <c r="H1" t="s">
-        <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
+      <c r="B2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>41</v>
       </c>
-      <c r="K1" t="s">
-        <v>42</v>
+      <c r="B3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -1070,7 +2039,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -1078,34 +2047,170 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>43</v>
+        <v>98</v>
       </c>
       <c r="C1" t="s">
-        <v>44</v>
+        <v>99</v>
       </c>
       <c r="D1" t="s">
-        <v>45</v>
+        <v>100</v>
       </c>
       <c r="E1" t="s">
-        <v>46</v>
+        <v>101</v>
       </c>
       <c r="F1" t="s">
+        <v>102</v>
+      </c>
+      <c r="G1" t="s">
+        <v>103</v>
+      </c>
+      <c r="H1" t="s">
+        <v>104</v>
+      </c>
+      <c r="I1" t="s">
+        <v>105</v>
+      </c>
+      <c r="J1" t="s">
+        <v>106</v>
+      </c>
+      <c r="K1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D2" t="s">
+        <v>110</v>
+      </c>
+      <c r="G2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D3" t="s">
+        <v>114</v>
+      </c>
+      <c r="G3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>47</v>
       </c>
-      <c r="G1" t="s">
-        <v>48</v>
-      </c>
-      <c r="H1" t="s">
-        <v>49</v>
-      </c>
-      <c r="I1" t="s">
-        <v>50</v>
-      </c>
-      <c r="J1" t="s">
-        <v>51</v>
-      </c>
-      <c r="K1" t="s">
-        <v>52</v>
+      <c r="B4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D4" t="s">
+        <v>118</v>
+      </c>
+      <c r="G4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" t="s">
+        <v>120</v>
+      </c>
+      <c r="C5" t="s">
+        <v>121</v>
+      </c>
+      <c r="D5" t="s">
+        <v>122</v>
+      </c>
+      <c r="G5" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D6" t="s">
+        <v>126</v>
+      </c>
+      <c r="G6" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" t="s">
+        <v>128</v>
+      </c>
+      <c r="C7" t="s">
+        <v>129</v>
+      </c>
+      <c r="D7" t="s">
+        <v>73</v>
+      </c>
+      <c r="G7" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" t="s">
+        <v>131</v>
+      </c>
+      <c r="C8" t="s">
+        <v>132</v>
+      </c>
+      <c r="D8" t="s">
+        <v>133</v>
+      </c>
+      <c r="G8" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" t="s">
+        <v>135</v>
+      </c>
+      <c r="C9" t="s">
+        <v>136</v>
+      </c>
+      <c r="D9" t="s">
+        <v>137</v>
+      </c>
+      <c r="G9" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -1116,7 +2221,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
@@ -1124,46 +2229,613 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F1" t="s">
+        <v>143</v>
+      </c>
+      <c r="G1" t="s">
+        <v>144</v>
+      </c>
+      <c r="H1" t="s">
+        <v>145</v>
+      </c>
+      <c r="I1" t="s">
+        <v>146</v>
+      </c>
+      <c r="J1" t="s">
+        <v>147</v>
+      </c>
+      <c r="K1" t="s">
+        <v>148</v>
+      </c>
+      <c r="L1" t="s">
+        <v>149</v>
+      </c>
+      <c r="M1" t="s">
+        <v>150</v>
+      </c>
+      <c r="N1" t="s">
+        <v>151</v>
+      </c>
+      <c r="O1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>153</v>
+      </c>
+      <c r="E2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G2">
+        <v>3923</v>
+      </c>
+      <c r="I2">
+        <v>2400</v>
+      </c>
+      <c r="M2">
+        <v>10200</v>
+      </c>
+      <c r="N2">
+        <v>40014600</v>
+      </c>
+      <c r="O2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E3" t="s">
+        <v>154</v>
+      </c>
+      <c r="G3">
+        <v>3959</v>
+      </c>
+      <c r="I3">
+        <v>2400</v>
+      </c>
+      <c r="M3">
+        <v>10200</v>
+      </c>
+      <c r="N3">
+        <v>40381800</v>
+      </c>
+      <c r="O3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" t="s">
+        <v>157</v>
+      </c>
+      <c r="E4" t="s">
+        <v>154</v>
+      </c>
+      <c r="G4">
+        <v>4894</v>
+      </c>
+      <c r="I4">
+        <v>2400</v>
+      </c>
+      <c r="M4">
+        <v>10200</v>
+      </c>
+      <c r="N4">
+        <v>49918800</v>
+      </c>
+      <c r="O4" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" t="s">
+        <v>158</v>
+      </c>
+      <c r="E5" t="s">
+        <v>159</v>
+      </c>
+      <c r="G5">
+        <v>4836</v>
+      </c>
+      <c r="I5">
+        <v>2400</v>
+      </c>
+      <c r="M5">
+        <v>10200</v>
+      </c>
+      <c r="N5">
+        <v>49327200</v>
+      </c>
+      <c r="O5" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" t="s">
+        <v>160</v>
+      </c>
+      <c r="E6" t="s">
+        <v>161</v>
+      </c>
+      <c r="G6">
+        <v>660</v>
+      </c>
+      <c r="H6">
+        <v>435</v>
+      </c>
+      <c r="M6">
+        <v>12000</v>
+      </c>
+      <c r="N6">
+        <v>7920000</v>
+      </c>
+      <c r="O6" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" t="s">
+        <v>162</v>
+      </c>
+      <c r="E7" t="s">
+        <v>163</v>
+      </c>
+      <c r="G7">
+        <v>1611</v>
+      </c>
+      <c r="M7">
+        <v>12000</v>
+      </c>
+      <c r="N7">
+        <v>19332000</v>
+      </c>
+      <c r="O7" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" t="s">
+        <v>164</v>
+      </c>
+      <c r="E8" t="s">
+        <v>165</v>
+      </c>
+      <c r="G8">
+        <v>2333</v>
+      </c>
+      <c r="M8">
+        <v>12000</v>
+      </c>
+      <c r="N8">
+        <v>27996000</v>
+      </c>
+      <c r="O8" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" t="s">
+        <v>166</v>
+      </c>
+      <c r="E9" t="s">
+        <v>167</v>
+      </c>
+      <c r="G9">
+        <v>1242</v>
+      </c>
+      <c r="M9">
+        <v>12000</v>
+      </c>
+      <c r="N9">
+        <v>14904000</v>
+      </c>
+      <c r="O9" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" t="s">
+        <v>168</v>
+      </c>
+      <c r="E10" t="s">
+        <v>169</v>
+      </c>
+      <c r="G10">
+        <v>1887</v>
+      </c>
+      <c r="M10">
+        <v>12000</v>
+      </c>
+      <c r="N10">
+        <v>22644000</v>
+      </c>
+      <c r="O10" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" t="s">
+        <v>170</v>
+      </c>
+      <c r="E11" t="s">
+        <v>171</v>
+      </c>
+      <c r="G11">
+        <v>2191</v>
+      </c>
+      <c r="M11">
+        <v>12000</v>
+      </c>
+      <c r="N11">
+        <v>26292000</v>
+      </c>
+      <c r="O11" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>53</v>
       </c>
-      <c r="C1" t="s">
-        <v>54</v>
-      </c>
-      <c r="D1" t="s">
-        <v>55</v>
-      </c>
-      <c r="E1" t="s">
-        <v>56</v>
-      </c>
-      <c r="F1" t="s">
-        <v>57</v>
-      </c>
-      <c r="G1" t="s">
-        <v>58</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="B12" t="s">
+        <v>172</v>
+      </c>
+      <c r="E12" t="s">
+        <v>161</v>
+      </c>
+      <c r="G12">
+        <v>715</v>
+      </c>
+      <c r="M12">
+        <v>11761</v>
+      </c>
+      <c r="N12">
+        <v>8409115</v>
+      </c>
+      <c r="O12" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13" t="s">
+        <v>173</v>
+      </c>
+      <c r="E13" t="s">
+        <v>167</v>
+      </c>
+      <c r="G13">
+        <v>1111</v>
+      </c>
+      <c r="M13">
+        <v>11761</v>
+      </c>
+      <c r="N13">
+        <v>13066471</v>
+      </c>
+      <c r="O13" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>53</v>
+      </c>
+      <c r="B14" t="s">
+        <v>174</v>
+      </c>
+      <c r="E14" t="s">
+        <v>163</v>
+      </c>
+      <c r="G14">
+        <v>1720</v>
+      </c>
+      <c r="M14">
+        <v>11761</v>
+      </c>
+      <c r="N14">
+        <v>20228920</v>
+      </c>
+      <c r="O14" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>59</v>
       </c>
-      <c r="I1" t="s">
-        <v>60</v>
-      </c>
-      <c r="J1" t="s">
-        <v>61</v>
-      </c>
-      <c r="K1" t="s">
-        <v>62</v>
-      </c>
-      <c r="L1" t="s">
-        <v>63</v>
-      </c>
-      <c r="M1" t="s">
-        <v>64</v>
-      </c>
-      <c r="N1" t="s">
+      <c r="B15" t="s">
+        <v>175</v>
+      </c>
+      <c r="E15" t="s">
+        <v>163</v>
+      </c>
+      <c r="G15">
+        <v>1389</v>
+      </c>
+      <c r="M15">
+        <v>9800</v>
+      </c>
+      <c r="N15">
+        <v>13612200</v>
+      </c>
+      <c r="O15" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>65</v>
       </c>
-      <c r="O1" t="s">
-        <v>66</v>
+      <c r="B16" t="s">
+        <v>176</v>
+      </c>
+      <c r="E16" t="s">
+        <v>167</v>
+      </c>
+      <c r="G16">
+        <v>1063</v>
+      </c>
+      <c r="M16">
+        <v>12300</v>
+      </c>
+      <c r="N16">
+        <v>13074900</v>
+      </c>
+      <c r="O16" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>65</v>
+      </c>
+      <c r="B17" t="s">
+        <v>177</v>
+      </c>
+      <c r="E17" t="s">
+        <v>163</v>
+      </c>
+      <c r="G17">
+        <v>1510</v>
+      </c>
+      <c r="M17">
+        <v>12300</v>
+      </c>
+      <c r="N17">
+        <v>18573000</v>
+      </c>
+      <c r="O17" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>70</v>
+      </c>
+      <c r="B18" t="s">
+        <v>178</v>
+      </c>
+      <c r="E18" t="s">
+        <v>161</v>
+      </c>
+      <c r="G18">
+        <v>753</v>
+      </c>
+      <c r="M18">
+        <v>10500</v>
+      </c>
+      <c r="N18">
+        <v>7906500</v>
+      </c>
+      <c r="O18" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>70</v>
+      </c>
+      <c r="B19" t="s">
+        <v>179</v>
+      </c>
+      <c r="E19" t="s">
+        <v>167</v>
+      </c>
+      <c r="G19">
+        <v>1268</v>
+      </c>
+      <c r="M19">
+        <v>10500</v>
+      </c>
+      <c r="N19">
+        <v>13314000</v>
+      </c>
+      <c r="O19" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" t="s">
+        <v>180</v>
+      </c>
+      <c r="E20" t="s">
+        <v>163</v>
+      </c>
+      <c r="G20">
+        <v>1733</v>
+      </c>
+      <c r="M20">
+        <v>10500</v>
+      </c>
+      <c r="N20">
+        <v>18196500</v>
+      </c>
+      <c r="O20" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>70</v>
+      </c>
+      <c r="B21" t="s">
+        <v>181</v>
+      </c>
+      <c r="E21" t="s">
+        <v>182</v>
+      </c>
+      <c r="G21">
+        <v>3336</v>
+      </c>
+      <c r="M21">
+        <v>10500</v>
+      </c>
+      <c r="N21">
+        <v>35028000</v>
+      </c>
+      <c r="O21" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>76</v>
+      </c>
+      <c r="B22" t="s">
+        <v>183</v>
+      </c>
+      <c r="E22" t="s">
+        <v>161</v>
+      </c>
+      <c r="G22">
+        <v>734</v>
+      </c>
+      <c r="M22">
+        <v>11500</v>
+      </c>
+      <c r="N22">
+        <v>8441000</v>
+      </c>
+      <c r="O22" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>76</v>
+      </c>
+      <c r="B23" t="s">
+        <v>184</v>
+      </c>
+      <c r="E23" t="s">
+        <v>167</v>
+      </c>
+      <c r="G23">
+        <v>1063</v>
+      </c>
+      <c r="M23">
+        <v>11500</v>
+      </c>
+      <c r="N23">
+        <v>12224500</v>
+      </c>
+      <c r="O23" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>76</v>
+      </c>
+      <c r="B24" t="s">
+        <v>185</v>
+      </c>
+      <c r="E24" t="s">
+        <v>163</v>
+      </c>
+      <c r="G24">
+        <v>1510</v>
+      </c>
+      <c r="M24">
+        <v>11500</v>
+      </c>
+      <c r="N24">
+        <v>17365000</v>
+      </c>
+      <c r="O24" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>76</v>
+      </c>
+      <c r="B25" t="s">
+        <v>186</v>
+      </c>
+      <c r="E25" t="s">
+        <v>165</v>
+      </c>
+      <c r="G25">
+        <v>2096</v>
+      </c>
+      <c r="M25">
+        <v>11500</v>
+      </c>
+      <c r="N25">
+        <v>24104000</v>
+      </c>
+      <c r="O25" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -1174,7 +2846,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AC1"/>
+  <dimension ref="A1:AC9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.25">
@@ -1182,88 +2854,248 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>67</v>
+        <v>187</v>
       </c>
       <c r="C1" t="s">
-        <v>68</v>
+        <v>188</v>
       </c>
       <c r="D1" t="s">
-        <v>69</v>
+        <v>189</v>
       </c>
       <c r="E1" t="s">
+        <v>190</v>
+      </c>
+      <c r="F1" t="s">
+        <v>191</v>
+      </c>
+      <c r="G1" t="s">
+        <v>192</v>
+      </c>
+      <c r="H1" t="s">
+        <v>193</v>
+      </c>
+      <c r="I1" t="s">
+        <v>194</v>
+      </c>
+      <c r="J1" t="s">
+        <v>195</v>
+      </c>
+      <c r="K1" t="s">
+        <v>196</v>
+      </c>
+      <c r="L1" t="s">
+        <v>197</v>
+      </c>
+      <c r="M1" t="s">
+        <v>198</v>
+      </c>
+      <c r="N1" t="s">
+        <v>199</v>
+      </c>
+      <c r="O1" t="s">
+        <v>200</v>
+      </c>
+      <c r="P1" t="s">
+        <v>201</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>202</v>
+      </c>
+      <c r="R1" t="s">
+        <v>203</v>
+      </c>
+      <c r="S1" t="s">
+        <v>204</v>
+      </c>
+      <c r="T1" t="s">
+        <v>205</v>
+      </c>
+      <c r="U1" t="s">
+        <v>206</v>
+      </c>
+      <c r="V1" t="s">
+        <v>207</v>
+      </c>
+      <c r="W1" t="s">
+        <v>208</v>
+      </c>
+      <c r="X1" t="s">
+        <v>209</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>210</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>211</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>212</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>213</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>215</v>
+      </c>
+      <c r="AC2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3">
+        <v>19</v>
+      </c>
+      <c r="C3">
+        <v>18</v>
+      </c>
+      <c r="D3">
+        <v>8</v>
+      </c>
+      <c r="G3" t="s">
+        <v>216</v>
+      </c>
+      <c r="AC3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4">
+        <v>10</v>
+      </c>
+      <c r="C4">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>5</v>
+      </c>
+      <c r="G4" t="s">
+        <v>217</v>
+      </c>
+      <c r="AC4">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>43</v>
+      </c>
+      <c r="D5">
+        <v>10</v>
+      </c>
+      <c r="G5" t="s">
+        <v>218</v>
+      </c>
+      <c r="AC5">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>26</v>
+      </c>
+      <c r="D6">
+        <v>8</v>
+      </c>
+      <c r="G6" t="s">
+        <v>219</v>
+      </c>
+      <c r="AC6">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7">
+        <v>28</v>
+      </c>
+      <c r="D7">
+        <v>8</v>
+      </c>
+      <c r="G7" t="s">
+        <v>220</v>
+      </c>
+      <c r="AC7">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>70</v>
       </c>
-      <c r="F1" t="s">
-        <v>71</v>
-      </c>
-      <c r="G1" t="s">
-        <v>72</v>
-      </c>
-      <c r="H1" t="s">
-        <v>73</v>
-      </c>
-      <c r="I1" t="s">
-        <v>74</v>
-      </c>
-      <c r="J1" t="s">
-        <v>75</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="B8">
+        <v>4</v>
+      </c>
+      <c r="C8">
+        <v>31</v>
+      </c>
+      <c r="D8">
+        <v>8</v>
+      </c>
+      <c r="G8" t="s">
+        <v>221</v>
+      </c>
+      <c r="AC8">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>76</v>
       </c>
-      <c r="L1" t="s">
-        <v>77</v>
-      </c>
-      <c r="M1" t="s">
-        <v>78</v>
-      </c>
-      <c r="N1" t="s">
-        <v>79</v>
-      </c>
-      <c r="O1" t="s">
+      <c r="B9">
+        <v>14</v>
+      </c>
+      <c r="C9">
+        <v>46</v>
+      </c>
+      <c r="D9">
+        <v>8</v>
+      </c>
+      <c r="G9" t="s">
+        <v>222</v>
+      </c>
+      <c r="AC9">
         <v>80</v>
-      </c>
-      <c r="P1" t="s">
-        <v>81</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>82</v>
-      </c>
-      <c r="R1" t="s">
-        <v>83</v>
-      </c>
-      <c r="S1" t="s">
-        <v>84</v>
-      </c>
-      <c r="T1" t="s">
-        <v>85</v>
-      </c>
-      <c r="U1" t="s">
-        <v>86</v>
-      </c>
-      <c r="V1" t="s">
-        <v>87</v>
-      </c>
-      <c r="W1" t="s">
-        <v>88</v>
-      </c>
-      <c r="X1" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>90</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>91</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>92</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>93</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1274,7 +3106,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -1282,16 +3114,128 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>95</v>
+        <v>223</v>
       </c>
       <c r="C1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E1" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>33</v>
       </c>
-      <c r="D1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E1" t="s">
-        <v>96</v>
+      <c r="B2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C2" t="s">
+        <v>226</v>
+      </c>
+      <c r="E2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" t="s">
+        <v>225</v>
+      </c>
+      <c r="C3" t="s">
+        <v>226</v>
+      </c>
+      <c r="E3" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" t="s">
+        <v>225</v>
+      </c>
+      <c r="C4" t="s">
+        <v>226</v>
+      </c>
+      <c r="E4" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" t="s">
+        <v>225</v>
+      </c>
+      <c r="C5" t="s">
+        <v>226</v>
+      </c>
+      <c r="E5" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6" t="s">
+        <v>225</v>
+      </c>
+      <c r="C6" t="s">
+        <v>226</v>
+      </c>
+      <c r="E6" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" t="s">
+        <v>225</v>
+      </c>
+      <c r="C7" t="s">
+        <v>226</v>
+      </c>
+      <c r="E7" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" t="s">
+        <v>225</v>
+      </c>
+      <c r="C8" t="s">
+        <v>226</v>
+      </c>
+      <c r="E8" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" t="s">
+        <v>225</v>
+      </c>
+      <c r="C9" t="s">
+        <v>226</v>
+      </c>
+      <c r="E9" t="s">
+        <v>234</v>
       </c>
     </row>
   </sheetData>
@@ -1310,16 +3254,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>95</v>
+        <v>223</v>
       </c>
       <c r="C1" t="s">
-        <v>33</v>
+        <v>81</v>
       </c>
       <c r="D1" t="s">
-        <v>97</v>
+        <v>235</v>
       </c>
       <c r="E1" t="s">
-        <v>98</v>
+        <v>236</v>
       </c>
     </row>
   </sheetData>
@@ -1338,16 +3282,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>81</v>
       </c>
       <c r="C1" t="s">
-        <v>99</v>
+        <v>237</v>
       </c>
       <c r="D1" t="s">
-        <v>100</v>
+        <v>238</v>
       </c>
       <c r="E1" t="s">
-        <v>101</v>
+        <v>239</v>
       </c>
     </row>
   </sheetData>
@@ -1366,10 +3310,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>81</v>
       </c>
       <c r="C1" t="s">
-        <v>102</v>
+        <v>240</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix schema NaN issue and fully update data mapper
</commit_message>
<xml_diff>
--- a/Populated_Parity_Template.xlsx
+++ b/Populated_Parity_Template.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="350">
   <si>
     <t>project_name</t>
   </si>
@@ -131,19 +131,31 @@
     <t>Admin</t>
   </si>
   <si>
-    <t>Hullahalli, Bengaluru</t>
+    <t>General Location: Hullahalli, Bengaluru. Key Road Access: Off, Begur - Koppa Rd, Hullahalli. Detailed Address (Legal): SY NO 41/4, AND SY NO 43/1, HULLAHALLI VILLAGE, JIGANI HOBLI, Anekal. Nearby Landmark: Near BVM Global School.</t>
+  </si>
+  <si>
+    <t>Bengaluru</t>
   </si>
   <si>
     <t>4 Acre</t>
   </si>
   <si>
-    <t>Lake-Facing Serenity</t>
+    <t>Lake-Facing Serenity and Vehicle-Free Zone. Focused on luxury, serene, lakefront living with all parking tucked underground.</t>
   </si>
   <si>
     <t>UnderConstruction</t>
   </si>
   <si>
-    <t>Villas</t>
+    <t>Villas (4 &amp; 5 BHK Villas)</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>₹ 10200 / Sq.ft Base</t>
+  </si>
+  <si>
+    <t>4BHK, 5BHK</t>
   </si>
   <si>
     <t>PRM/KA/RERA/1251/308/PR/190325/007593</t>
@@ -152,589 +164,763 @@
     <t>SOBHA Neopolis</t>
   </si>
   <si>
+    <t>Panathur, Off Marathahalli-ORR, Bengaluru</t>
+  </si>
+  <si>
+    <t>25 Acres 35.9 Guntas</t>
+  </si>
+  <si>
+    <t>Greek / Santorini Theme</t>
+  </si>
+  <si>
+    <t>Premium Residential Township</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>₹ 12000 / Sq.ft Base</t>
+  </si>
+  <si>
+    <t>1 BHK, 3 BHK, 3+Study, 4 BHK</t>
+  </si>
+  <si>
+    <t>PRM/KA/RERA/1251/446/PR/200923/006269, 6270, 6271</t>
+  </si>
+  <si>
+    <t>Godrej Woods</t>
+  </si>
+  <si>
+    <t>Thanisandra Main Road, Near Kogilu Cross, North Bengaluru</t>
+  </si>
+  <si>
+    <t>~7 Acres</t>
+  </si>
+  <si>
+    <t>Sanctuary in the City (Forest-themed living with 1600+ trees)</t>
+  </si>
+  <si>
+    <t>High-Rise Residential Apartments (Forest-Themed)</t>
+  </si>
+  <si>
+    <t>New Launch / Pre-Launch Phase</t>
+  </si>
+  <si>
+    <t>2 BHK, 3 BHK Premium, 3 BHK Luxe</t>
+  </si>
+  <si>
+    <t>PRM/KA/RERA/1251/472/PR/121125/008248</t>
+  </si>
+  <si>
+    <t>Brigade Belvedere</t>
+  </si>
+  <si>
+    <t>Budigere Road, Bengaluru</t>
+  </si>
+  <si>
+    <t>~10.75 Acres</t>
+  </si>
+  <si>
+    <t>Premium High-Rise Urban Living</t>
+  </si>
+  <si>
+    <t>Residential Apartments</t>
+  </si>
+  <si>
+    <t>Phase 1 | 775 Availabe Units | Tower A &amp; B</t>
+  </si>
+  <si>
+    <t>₹ 11761 / Sq.ft Base</t>
+  </si>
+  <si>
+    <t>1 BHK, 2 BHK, 2 B2T, 3 B3T, 3.5BHK</t>
+  </si>
+  <si>
+    <t>PRM/KA/RERA/1251/446/PR/240326/008549</t>
+  </si>
+  <si>
+    <t>Bren Aspera</t>
+  </si>
+  <si>
+    <t>Old Madras Road, Bengaluru</t>
+  </si>
+  <si>
+    <t>4.39 Acres (~4 Acres 15 Gunthas)</t>
+  </si>
+  <si>
+    <t>Premium Community Living with Brennovation Features</t>
+  </si>
+  <si>
+    <t>Premium Residential Apartments (3 BHK Only)</t>
+  </si>
+  <si>
+    <t>Active Inventory in Both Towers</t>
+  </si>
+  <si>
+    <t>₹ 9800 / Sq.ft Base</t>
+  </si>
+  <si>
+    <t>3 BHK Only</t>
+  </si>
+  <si>
+    <t>PRM/KA/RERA/1251/310/PR/300622/005028</t>
+  </si>
+  <si>
+    <t>Godrej Parkshire</t>
+  </si>
+  <si>
+    <t>Sarkariguttahalli Village, Kasaba Hobli, Hosakote, Bengaluru Rural</t>
+  </si>
+  <si>
+    <t>13.8 Acres</t>
+  </si>
+  <si>
+    <t>Born Green | Nature-Themed High-Rise Living</t>
+  </si>
+  <si>
+    <t>Premium Residential Apartments</t>
+  </si>
+  <si>
+    <t>2 BHK &amp; 3 BHK Homes</t>
+  </si>
+  <si>
+    <t>₹ 12300 / Sq.ft Base</t>
+  </si>
+  <si>
+    <t>2 BHK Premium, 2 BHK Luxe, 3 BHK Premium, 3 BHK Luxe</t>
+  </si>
+  <si>
+    <t>PRM/KA/RERA/1250/304/PR/090126/008393</t>
+  </si>
+  <si>
+    <t>Sattva Songbird</t>
+  </si>
+  <si>
+    <t>Budigere Main Road, off Old Madras Road, Bengaluru</t>
+  </si>
+  <si>
+    <t>16 Acres</t>
+  </si>
+  <si>
+    <t>Nature-Themed Township Living</t>
+  </si>
+  <si>
+    <t>Integrated Township (Apartments + Row Houses)</t>
+  </si>
+  <si>
+    <t>Phase 2 (Pre-Launch)</t>
+  </si>
+  <si>
+    <t>₹ 10500 / Sq.ft Base</t>
+  </si>
+  <si>
+    <t>Studio, 1, 2, 2.5, 3 BHK + Row Houses | Phase 2: 2 &amp; 3 BHK</t>
+  </si>
+  <si>
+    <t>Phase 2: PRM/KA/RERA/1251/310/PR/270326/008557</t>
+  </si>
+  <si>
+    <t>SOBHA OneWorld</t>
+  </si>
+  <si>
+    <t>Along Old Madras Road near Hoskote Toll Gate, Bengaluru</t>
+  </si>
+  <si>
+    <t>48 Acres | 15.32 Guntas</t>
+  </si>
+  <si>
+    <t>Next-generation integrated township</t>
+  </si>
+  <si>
+    <t>Integrated Township with Residential, Retail &amp; Commercial Spaces</t>
+  </si>
+  <si>
+    <t>Residential wings</t>
+  </si>
+  <si>
+    <t>₹ 11500 / Sq.ft Base</t>
+  </si>
+  <si>
+    <t>1 BHK, 2 BHK Luxe, 2 BHK Grande, 3 BHK Luxe, 3 BHK Grande, 4 BHK Luxe, 4 BHK Grande</t>
+  </si>
+  <si>
+    <t>Not specified</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>logo_url</t>
+  </si>
+  <si>
+    <t>website</t>
+  </si>
+  <si>
+    <t>buildergrade</t>
+  </si>
+  <si>
+    <t>corporate_rera</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>reputation</t>
+  </si>
+  <si>
+    <t>years_in_market</t>
+  </si>
+  <si>
+    <t>past_projects</t>
+  </si>
+  <si>
+    <t>financial_strength</t>
+  </si>
+  <si>
+    <t>Rainbow Properties</t>
+  </si>
+  <si>
+    <t>Construction Quality: 1,456 quality checks, backward integrated | Feedback: Positive testimonials included</t>
+  </si>
+  <si>
+    <t>Premium</t>
+  </si>
+  <si>
+    <t>Strong - in-house manufacturing</t>
+  </si>
+  <si>
+    <t>SOBHA Limited</t>
+  </si>
+  <si>
+    <t>Construction Quality: High (Mivan Technology usually employed); ISO certified processes. | Feedback: Generally positive regarding amenities and landscape. Some mixed reviews regarding handover timelines in past projects.</t>
+  </si>
+  <si>
+    <t>Premium national developer</t>
+  </si>
+  <si>
+    <t>530+ projects</t>
+  </si>
+  <si>
+    <t>Very Strong (Publicly Listed: GODREJPROP); High liquidity and land bank.</t>
+  </si>
+  <si>
+    <t>Godrej Properties Limited</t>
+  </si>
+  <si>
+    <t>Construction Quality: High (Mivan Technology) | Feedback: Generally positive</t>
+  </si>
+  <si>
+    <t>Tier-1 Developer; India's No. 1 listed real estate developer by sales booking. High brand recall.</t>
+  </si>
+  <si>
+    <t>Godrej Woodsman Estate, Godrej Platinum, Godrej Air, Godrej Reserve</t>
+  </si>
+  <si>
+    <t>Strong</t>
+  </si>
+  <si>
+    <t>Brigade Group</t>
+  </si>
+  <si>
+    <t>Construction Quality: High (Aluminium Formwork Technology) | Feedback: Generally Positive</t>
+  </si>
+  <si>
+    <t>Tier-1 builder (Brigade)</t>
+  </si>
+  <si>
+    <t>Brigade Gateway, Brigade Exotica, etc.</t>
+  </si>
+  <si>
+    <t>Strong Mid-Tier Developer</t>
+  </si>
+  <si>
+    <t>Bren Corporation Pvt. Ltd.</t>
+  </si>
+  <si>
+    <t>Construction Quality: High | Feedback: Generally positive</t>
+  </si>
+  <si>
+    <t>Established Premium Bangalore Developer</t>
+  </si>
+  <si>
+    <t>Avalon, Unity, Paddington, Trillium, Celestia, Edgewaters, Zahara, Northern Lights</t>
+  </si>
+  <si>
+    <t>Godrej Properties Ltd.</t>
+  </si>
+  <si>
+    <t>Construction Quality: Premium | Feedback: Generally Positive</t>
+  </si>
+  <si>
+    <t>Tier-1 national developer</t>
+  </si>
+  <si>
+    <t>Godrej Air, Godrej United, Godrej Splendour, Godrej Woodscape, Godrej Park Retreat etc.</t>
+  </si>
+  <si>
+    <t>Strong (CRISIL A Rated)</t>
+  </si>
+  <si>
+    <t>Sattva Group / Sattva Resi Pvt. Ltd.</t>
+  </si>
+  <si>
+    <t>Construction Quality: Premium SOBHA construction quality | Feedback: Generally positive</t>
+  </si>
+  <si>
+    <t>Tier-1 Bangalore Developer</t>
+  </si>
+  <si>
+    <t>Sattva Greenage, Magnificia, Luxuria, Divinity, Park Cubix</t>
+  </si>
+  <si>
+    <t>Strong listed developer</t>
+  </si>
+  <si>
+    <t>Construction Quality: Premium | Feedback: Generally positive</t>
+  </si>
+  <si>
+    <t>Tier-1 premium developer</t>
+  </si>
+  <si>
+    <t>SOBHA Dream Acres, SOBHA City, SOBHA Windsor, SOBHA Royal Pavilion</t>
+  </si>
+  <si>
+    <t>pros</t>
+  </si>
+  <si>
+    <t>cons</t>
+  </si>
+  <si>
+    <t>usp</t>
+  </si>
+  <si>
+    <t>usp_highlights</t>
+  </si>
+  <si>
+    <t>closing_pitch</t>
+  </si>
+  <si>
+    <t>target_customer</t>
+  </si>
+  <si>
+    <t>objection_handling</t>
+  </si>
+  <si>
+    <t>legal_notes</t>
+  </si>
+  <si>
+    <t>timeline_risk</t>
+  </si>
+  <si>
+    <t>overall_rating</t>
+  </si>
+  <si>
+    <t>["Brand, open space, amenities, location"]</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>Brand, open space, amenities, location</t>
+  </si>
+  <si>
+    <t>IT professionals, families</t>
+  </si>
+  <si>
+    <t>["1. Brand: Godrej Trust. 2. Theme: Forest Living (Unique in N. Blr). 3. Low Density: Only ~550 units on 7 acres. 4. Location: Right on Main Road, near upcoming Metro."]</t>
+  </si>
+  <si>
+    <t>1. Brand: Godrej Trust. 2. Theme: Forest Living (Unique in N. Blr). 3. Low Density: Only ~550 units on 7 acres. 4. Location: Right on Main Road, near upcoming Metro.</t>
+  </si>
+  <si>
+    <t>IT Professionals (VP/Director level) working in Manyata, Doctors (Aster/Cytecare), Investors.</t>
+  </si>
+  <si>
+    <t>["1. On mainroad 2. Price is decent 3. Only 2 Phases for sales 4. High Rise - 43 floors 5. Opp to Godrej woodestates - Soldout"]</t>
+  </si>
+  <si>
+    <t>1. On mainroad 2. Price is decent 3. Only 2 Phases for sales 4. High Rise - 43 floors 5. Opp to Godrej woodestates - Soldout</t>
+  </si>
+  <si>
+    <t>IT families</t>
+  </si>
+  <si>
+    <t>["Prime location; low density; large units"]</t>
+  </si>
+  <si>
+    <t>Prime location; low density; large units</t>
+  </si>
+  <si>
+    <t>IT professionals, investors, upgrade buyers, Whitefield workforce, long-term appreciation buyers</t>
+  </si>
+  <si>
+    <t>["Godrej brand; 13.8 acres; 80% open space; 32,500 sqft clubhouse; Whitefield-Hoskote growth belt; 1% payment plan; strong future appreciation"]</t>
+  </si>
+  <si>
+    <t>Godrej brand; 13.8 acres; 80% open space; 32,500 sqft clubhouse; Whitefield-Hoskote growth belt; 1% payment plan; strong future appreciation</t>
+  </si>
+  <si>
+    <t>IT Professionals + Investors</t>
+  </si>
+  <si>
+    <t>["16 Acres Township | Sattva Brand | 80% Open Space | STRR Growth"]</t>
+  </si>
+  <si>
+    <t>16 Acres Township | Sattva Brand | 80% Open Space | STRR Growth</t>
+  </si>
+  <si>
+    <t>Investors, IT professionals, upgrade buyers, township lifestyle buyers, East Bengaluru growth buyers</t>
+  </si>
+  <si>
+    <t>["SOBHA brand, 48-acre township, 3,484 units, 14 wings, OMR frontage, strong STRR connectivity, multiple unit options"]</t>
+  </si>
+  <si>
+    <t>SOBHA brand, 48-acre township, 3,484 units, 14 wings, OMR frontage, strong STRR connectivity, multiple unit options</t>
+  </si>
+  <si>
+    <t>Investors + End Users</t>
+  </si>
+  <si>
+    <t>["Brand, Township"]</t>
+  </si>
+  <si>
+    <t>Brand, Township</t>
+  </si>
+  <si>
+    <t>Investors, East Bengaluru buyers, IT professionals, premium township buyers</t>
+  </si>
+  <si>
+    <t>unitnumber</t>
+  </si>
+  <si>
+    <t>tower</t>
+  </si>
+  <si>
+    <t>floornumber</t>
+  </si>
+  <si>
+    <t>config</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>actualsba</t>
+  </si>
+  <si>
+    <t>carpetarea</t>
+  </si>
+  <si>
+    <t>udsarea</t>
+  </si>
+  <si>
+    <t>facing</t>
+  </si>
+  <si>
+    <t>wccount</t>
+  </si>
+  <si>
+    <t>balconycount</t>
+  </si>
+  <si>
+    <t>pricepersqft</t>
+  </si>
+  <si>
+    <t>pricetotal</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>U-1</t>
+  </si>
+  <si>
+    <t>4BHK</t>
+  </si>
+  <si>
+    <t>Available</t>
+  </si>
+  <si>
+    <t>U-2</t>
+  </si>
+  <si>
+    <t>U-3</t>
+  </si>
+  <si>
+    <t>U-4</t>
+  </si>
+  <si>
+    <t>5BHK</t>
+  </si>
+  <si>
+    <t>U-5</t>
+  </si>
+  <si>
+    <t>1 BHK</t>
+  </si>
+  <si>
+    <t>U-6</t>
+  </si>
+  <si>
+    <t>3 BHK</t>
+  </si>
+  <si>
+    <t>U-7</t>
+  </si>
+  <si>
+    <t>4 BHK</t>
+  </si>
+  <si>
+    <t>U-8</t>
+  </si>
+  <si>
+    <t>2 BHK</t>
+  </si>
+  <si>
+    <t>U-9</t>
+  </si>
+  <si>
+    <t>U-10</t>
+  </si>
+  <si>
+    <t>3 BHK Luxe</t>
+  </si>
+  <si>
+    <t>U-11</t>
+  </si>
+  <si>
+    <t>U-12</t>
+  </si>
+  <si>
+    <t>U-13</t>
+  </si>
+  <si>
+    <t>U-14</t>
+  </si>
+  <si>
+    <t>U-15</t>
+  </si>
+  <si>
+    <t>U-16</t>
+  </si>
+  <si>
+    <t>U-17</t>
+  </si>
+  <si>
+    <t>U-18</t>
+  </si>
+  <si>
+    <t>U-19</t>
+  </si>
+  <si>
+    <t>U-20</t>
+  </si>
+  <si>
+    <t>Row House</t>
+  </si>
+  <si>
+    <t>U-21</t>
+  </si>
+  <si>
+    <t>U-22</t>
+  </si>
+  <si>
+    <t>U-23</t>
+  </si>
+  <si>
+    <t>U-24</t>
+  </si>
+  <si>
+    <t>no_of_towers</t>
+  </si>
+  <si>
+    <t>floors_per_tower</t>
+  </si>
+  <si>
+    <t>units_per_floor</t>
+  </si>
+  <si>
+    <t>elevators_per_tower</t>
+  </si>
+  <si>
+    <t>service_elevators_per_tower</t>
+  </si>
+  <si>
+    <t>construction_type</t>
+  </si>
+  <si>
+    <t>structure_details</t>
+  </si>
+  <si>
+    <t>wall_finishing_interior</t>
+  </si>
+  <si>
+    <t>wall_finishing_exterior</t>
+  </si>
+  <si>
+    <t>flooring_living_dining</t>
+  </si>
+  <si>
+    <t>flooring_master_bedroom</t>
+  </si>
+  <si>
+    <t>flooring_other_bedrooms</t>
+  </si>
+  <si>
+    <t>flooring_balcony_utility</t>
+  </si>
+  <si>
+    <t>kitchen_countertop</t>
+  </si>
+  <si>
+    <t>kitchen_sink_details</t>
+  </si>
+  <si>
+    <t>kitchen_dado_tiling</t>
+  </si>
+  <si>
+    <t>gas_pipeline_provision</t>
+  </si>
+  <si>
+    <t>bathroom_sanitary_ware</t>
+  </si>
+  <si>
+    <t>bathroom_cp_fittings</t>
+  </si>
+  <si>
+    <t>bathroom_dado_tiling</t>
+  </si>
+  <si>
+    <t>main_door_specs</t>
+  </si>
+  <si>
+    <t>internal_doors_specs</t>
+  </si>
+  <si>
+    <t>windows_specs</t>
+  </si>
+  <si>
+    <t>electrical_switches</t>
+  </si>
+  <si>
+    <t>power_backup</t>
+  </si>
+  <si>
+    <t>road_width</t>
+  </si>
+  <si>
+    <t>water_source</t>
+  </si>
+  <si>
+    <t>open_space_pct</t>
+  </si>
+  <si>
+    <t>Seismic-II zone compliant RCC framed structure | Row Houses/Villas</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>RCC-framed high-rise structure, Neo-classical / Greek-inspired architectural design</t>
+  </si>
+  <si>
+    <t>78</t>
+  </si>
+  <si>
+    <t>RCC Framed Structure (Aluminum Formwork / Shear Wall Technology).</t>
+  </si>
+  <si>
+    <t>76</t>
+  </si>
+  <si>
+    <t>RCC High-rise</t>
+  </si>
+  <si>
+    <t>81</t>
+  </si>
+  <si>
+    <t>RCC (Aluminium Formwork)</t>
+  </si>
+  <si>
+    <t>RCC High-Rise Structure</t>
+  </si>
+  <si>
+    <t>80</t>
+  </si>
+  <si>
+    <t>RCC / Shear Wall Structure</t>
+  </si>
+  <si>
+    <t>High-rise residential township</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>size_specs</t>
+  </si>
+  <si>
+    <t>Clubhouse</t>
+  </si>
+  <si>
+    <t>Main Clubhouse</t>
+  </si>
+  <si>
+    <t>11000</t>
+  </si>
+  <si>
+    <t>77850</t>
+  </si>
+  <si>
+    <t>20000</t>
+  </si>
+  <si>
+    <t>25000</t>
+  </si>
+  <si>
+    <t>15000</t>
+  </si>
+  <si>
+    <t>32500</t>
+  </si>
+  <si>
+    <t>100000</t>
+  </si>
+  <si>
+    <t>50000</t>
+  </si>
+  <si>
+    <t>distance_km</t>
+  </si>
+  <si>
+    <t>travel_time</t>
+  </si>
+  <si>
+    <t>General</t>
+  </si>
+  <si>
+    <t>Lakefront living; Close to Bannerghatta Road; Near Kalena Agrahara Metro Station (6 km) and Wipro Limited (5 km)</t>
+  </si>
+  <si>
     <t>Panathur Main Road, ORR IT Corridor</t>
   </si>
   <si>
-    <t>25 Acres</t>
-  </si>
-  <si>
-    <t>Greek / Santorini Theme</t>
-  </si>
-  <si>
-    <t>Premium Residential Township</t>
-  </si>
-  <si>
-    <t>PRM/KA/RERA/1251/446/PR/200923/006269</t>
-  </si>
-  <si>
-    <t>Godrej Woods</t>
-  </si>
-  <si>
-    <t>Thanisandra Main Road</t>
-  </si>
-  <si>
-    <t>7 Acres</t>
-  </si>
-  <si>
-    <t>Forest-Themed</t>
-  </si>
-  <si>
-    <t>High-Rise Residential Apartments</t>
-  </si>
-  <si>
-    <t>PRM/KA/RERA/1251/472/PR/121125/008248</t>
-  </si>
-  <si>
-    <t>Brigade Belvedere</t>
-  </si>
-  <si>
-    <t>Budigere Cross</t>
-  </si>
-  <si>
-    <t>10.75 Acres</t>
-  </si>
-  <si>
-    <t>Premium High-Rise Urban Living</t>
-  </si>
-  <si>
-    <t>Residential Apartments</t>
-  </si>
-  <si>
-    <t>PRM/KA/RERA/1251/446/PR/240326/008549</t>
-  </si>
-  <si>
-    <t>Bren Aspera</t>
+    <t>Near Bhartiya City / Reva University</t>
+  </si>
+  <si>
+    <t>Budigere Cross, Near Old Madras Road</t>
   </si>
   <si>
     <t>Old Madras Road Corridor</t>
   </si>
   <si>
-    <t>4.39 Acres</t>
-  </si>
-  <si>
-    <t>Premium Community Living</t>
-  </si>
-  <si>
-    <t>Premium Residential Apartments</t>
-  </si>
-  <si>
-    <t>PRM/KA/RERA/1251/310/PR/300622/005028</t>
-  </si>
-  <si>
-    <t>Godrej Parkshire</t>
-  </si>
-  <si>
-    <t>Hoskote</t>
-  </si>
-  <si>
-    <t>13.8 Acres</t>
-  </si>
-  <si>
-    <t>Nature-Themed High-Rise Living</t>
-  </si>
-  <si>
-    <t>PRM/KA/RERA/1250/304/PR/090126/008393</t>
-  </si>
-  <si>
-    <t>Sattva Songbird</t>
-  </si>
-  <si>
-    <t>300 meters from Old Madras Road</t>
-  </si>
-  <si>
-    <t>16 Acres</t>
-  </si>
-  <si>
-    <t>Nature-Themed Township Living</t>
-  </si>
-  <si>
-    <t>Integrated Township</t>
-  </si>
-  <si>
-    <t>PRM/KA/RERA/1251/310/PR/270326/008557</t>
-  </si>
-  <si>
-    <t>SOBHA OneWorld</t>
-  </si>
-  <si>
-    <t>Old Madras Road</t>
-  </si>
-  <si>
-    <t>48 Acres</t>
-  </si>
-  <si>
-    <t>Next-generation integrated township</t>
-  </si>
-  <si>
-    <t>Pending</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>logo_url</t>
-  </si>
-  <si>
-    <t>website</t>
-  </si>
-  <si>
-    <t>buildergrade</t>
-  </si>
-  <si>
-    <t>corporate_rera</t>
-  </si>
-  <si>
-    <t>description</t>
-  </si>
-  <si>
-    <t>reputation</t>
-  </si>
-  <si>
-    <t>years_in_market</t>
-  </si>
-  <si>
-    <t>past_projects</t>
-  </si>
-  <si>
-    <t>financial_strength</t>
-  </si>
-  <si>
-    <t>Rainbow Properties</t>
-  </si>
-  <si>
-    <t>SOBHA Limited</t>
-  </si>
-  <si>
-    <t>Godrej Properties Limited</t>
-  </si>
-  <si>
-    <t>Brigade Group</t>
-  </si>
-  <si>
-    <t>Bren Corporation Pvt. Ltd.</t>
-  </si>
-  <si>
-    <t>Godrej Properties Ltd.</t>
-  </si>
-  <si>
-    <t>Sattva Group</t>
-  </si>
-  <si>
-    <t>pros</t>
-  </si>
-  <si>
-    <t>cons</t>
-  </si>
-  <si>
-    <t>usp</t>
-  </si>
-  <si>
-    <t>usp_highlights</t>
-  </si>
-  <si>
-    <t>closing_pitch</t>
-  </si>
-  <si>
-    <t>target_customer</t>
-  </si>
-  <si>
-    <t>objection_handling</t>
-  </si>
-  <si>
-    <t>legal_notes</t>
-  </si>
-  <si>
-    <t>timeline_risk</t>
-  </si>
-  <si>
-    <t>overall_rating</t>
-  </si>
-  <si>
-    <t>["Lakefront living","Vehicle-Free Zone","Large UDS"]</t>
-  </si>
-  <si>
-    <t>["Common wall structure","Far from metro"]</t>
-  </si>
-  <si>
-    <t>Lakefront living</t>
-  </si>
-  <si>
-    <t>IT professionals, families</t>
-  </si>
-  <si>
-    <t>["Theme: Greek Santorini","3 Clubhouses","Low Density"]</t>
-  </si>
-  <si>
-    <t>["High pricing","Traffic on Panathur road"]</t>
-  </si>
-  <si>
-    <t>Theme: Greek Santorini</t>
-  </si>
-  <si>
-    <t>IT Professionals (VP/Director level)</t>
-  </si>
-  <si>
-    <t>["Forest Living","Main Road Location"]</t>
-  </si>
-  <si>
-    <t>["Small 2BHK size"]</t>
-  </si>
-  <si>
-    <t>Forest Living</t>
-  </si>
-  <si>
-    <t>IT families</t>
-  </si>
-  <si>
-    <t>["High Rise 43 floors","Large units","Prime location"]</t>
-  </si>
-  <si>
-    <t>[]</t>
-  </si>
-  <si>
-    <t>High Rise 43 floors</t>
-  </si>
-  <si>
-    <t>IT professionals, investors</t>
-  </si>
-  <si>
-    <t>["Low density","Established builder"]</t>
-  </si>
-  <si>
-    <t>["Only 3BHK available"]</t>
-  </si>
-  <si>
-    <t>Low density</t>
-  </si>
-  <si>
-    <t>IT Professionals + Investors</t>
-  </si>
-  <si>
-    <t>["Nature-Themed Township Living","Godrej brand","Large land parcel"]</t>
-  </si>
-  <si>
-    <t>["Hoskote distance"]</t>
-  </si>
-  <si>
-    <t>Investors, IT professionals</t>
-  </si>
-  <si>
-    <t>["16 Acres Township","Sattva Brand","STRR Growth"]</t>
-  </si>
-  <si>
-    <t>["Long Timeline"]</t>
-  </si>
-  <si>
-    <t>16 Acres Township</t>
-  </si>
-  <si>
-    <t>Investors + End Users</t>
-  </si>
-  <si>
-    <t>["SOBHA brand","48-acre township","Multiple unit options"]</t>
-  </si>
-  <si>
-    <t>["Possession details not shared"]</t>
-  </si>
-  <si>
-    <t>SOBHA brand</t>
-  </si>
-  <si>
-    <t>Investors, East Bengaluru buyers</t>
-  </si>
-  <si>
-    <t>unitnumber</t>
-  </si>
-  <si>
-    <t>tower</t>
-  </si>
-  <si>
-    <t>floornumber</t>
-  </si>
-  <si>
-    <t>config</t>
-  </si>
-  <si>
-    <t>type</t>
-  </si>
-  <si>
-    <t>actualsba</t>
-  </si>
-  <si>
-    <t>carpetarea</t>
-  </si>
-  <si>
-    <t>udsarea</t>
-  </si>
-  <si>
-    <t>facing</t>
-  </si>
-  <si>
-    <t>wccount</t>
-  </si>
-  <si>
-    <t>balconycount</t>
-  </si>
-  <si>
-    <t>pricepersqft</t>
-  </si>
-  <si>
-    <t>pricetotal</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>U-1</t>
-  </si>
-  <si>
-    <t>4BHK</t>
-  </si>
-  <si>
-    <t>Available</t>
-  </si>
-  <si>
-    <t>U-2</t>
-  </si>
-  <si>
-    <t>U-3</t>
-  </si>
-  <si>
-    <t>U-4</t>
-  </si>
-  <si>
-    <t>5BHK</t>
-  </si>
-  <si>
-    <t>U-5</t>
-  </si>
-  <si>
-    <t>1 BHK</t>
-  </si>
-  <si>
-    <t>U-6</t>
-  </si>
-  <si>
-    <t>3 BHK</t>
-  </si>
-  <si>
-    <t>U-7</t>
-  </si>
-  <si>
-    <t>4 BHK</t>
-  </si>
-  <si>
-    <t>U-8</t>
-  </si>
-  <si>
-    <t>2 BHK</t>
-  </si>
-  <si>
-    <t>U-9</t>
-  </si>
-  <si>
-    <t>3 BHK Premium</t>
-  </si>
-  <si>
-    <t>U-10</t>
-  </si>
-  <si>
-    <t>3 BHK Luxe</t>
-  </si>
-  <si>
-    <t>U-11</t>
-  </si>
-  <si>
-    <t>U-12</t>
-  </si>
-  <si>
-    <t>U-13</t>
-  </si>
-  <si>
-    <t>U-14</t>
-  </si>
-  <si>
-    <t>U-15</t>
-  </si>
-  <si>
-    <t>U-16</t>
-  </si>
-  <si>
-    <t>U-17</t>
-  </si>
-  <si>
-    <t>U-18</t>
-  </si>
-  <si>
-    <t>U-19</t>
-  </si>
-  <si>
-    <t>U-20</t>
-  </si>
-  <si>
-    <t>Row House</t>
-  </si>
-  <si>
-    <t>U-21</t>
-  </si>
-  <si>
-    <t>U-22</t>
-  </si>
-  <si>
-    <t>U-23</t>
-  </si>
-  <si>
-    <t>U-24</t>
-  </si>
-  <si>
-    <t>no_of_towers</t>
-  </si>
-  <si>
-    <t>floors_per_tower</t>
-  </si>
-  <si>
-    <t>units_per_floor</t>
-  </si>
-  <si>
-    <t>elevators_per_tower</t>
-  </si>
-  <si>
-    <t>service_elevators_per_tower</t>
-  </si>
-  <si>
-    <t>construction_type</t>
-  </si>
-  <si>
-    <t>structure_details</t>
-  </si>
-  <si>
-    <t>wall_finishing_interior</t>
-  </si>
-  <si>
-    <t>wall_finishing_exterior</t>
-  </si>
-  <si>
-    <t>flooring_living_dining</t>
-  </si>
-  <si>
-    <t>flooring_master_bedroom</t>
-  </si>
-  <si>
-    <t>flooring_other_bedrooms</t>
-  </si>
-  <si>
-    <t>flooring_balcony_utility</t>
-  </si>
-  <si>
-    <t>kitchen_countertop</t>
-  </si>
-  <si>
-    <t>kitchen_sink_details</t>
-  </si>
-  <si>
-    <t>kitchen_dado_tiling</t>
-  </si>
-  <si>
-    <t>gas_pipeline_provision</t>
-  </si>
-  <si>
-    <t>bathroom_sanitary_ware</t>
-  </si>
-  <si>
-    <t>bathroom_cp_fittings</t>
-  </si>
-  <si>
-    <t>bathroom_dado_tiling</t>
-  </si>
-  <si>
-    <t>main_door_specs</t>
-  </si>
-  <si>
-    <t>internal_doors_specs</t>
-  </si>
-  <si>
-    <t>windows_specs</t>
-  </si>
-  <si>
-    <t>electrical_switches</t>
-  </si>
-  <si>
-    <t>power_backup</t>
-  </si>
-  <si>
-    <t>road_width</t>
-  </si>
-  <si>
-    <t>water_source</t>
-  </si>
-  <si>
-    <t>open_space_pct</t>
-  </si>
-  <si>
-    <t>Seismic-II zone compliant RCC framed structure</t>
-  </si>
-  <si>
-    <t>RCC-framed high-rise structure</t>
-  </si>
-  <si>
-    <t>RCC Framed Structure</t>
-  </si>
-  <si>
-    <t>RCC High-rise</t>
-  </si>
-  <si>
-    <t>RCC (Aluminium Formwork)</t>
-  </si>
-  <si>
-    <t>RCC High-Rise Structure</t>
-  </si>
-  <si>
-    <t>RCC / Shear Wall Structure</t>
-  </si>
-  <si>
-    <t>High-rise residential township</t>
-  </si>
-  <si>
-    <t>category</t>
-  </si>
-  <si>
-    <t>size_specs</t>
-  </si>
-  <si>
-    <t>Clubhouse</t>
-  </si>
-  <si>
-    <t>Main Clubhouse</t>
-  </si>
-  <si>
-    <t>11,000 Sq.ft</t>
-  </si>
-  <si>
-    <t>77,850 sq ft</t>
-  </si>
-  <si>
-    <t>20,000 Sq. Ft.</t>
-  </si>
-  <si>
-    <t>25,000 Sq.ft</t>
-  </si>
-  <si>
-    <t>15,000 Sq.ft</t>
-  </si>
-  <si>
-    <t>32,500 sq.ft</t>
-  </si>
-  <si>
-    <t>100,000 sqft</t>
-  </si>
-  <si>
-    <t>50,000 sqft</t>
-  </si>
-  <si>
-    <t>distance_km</t>
-  </si>
-  <si>
-    <t>travel_time</t>
+    <t>Hoskote | Whitefield-Hoskote Road | Hope Farm Soukya Road Extension</t>
+  </si>
+  <si>
+    <t>300 meters from Old Madras Road (OMR)</t>
+  </si>
+  <si>
+    <t>Old Madras Road, Whitefield-Hoskote Road, Budigere Road, STRR</t>
   </si>
   <si>
     <t>amount</t>
@@ -767,52 +953,85 @@
     <t>1 Kms</t>
   </si>
   <si>
-    <t>45-60 km</t>
+    <t>45 - 60 km (Kempegowda International Airport - BLR)</t>
+  </si>
+  <si>
+    <t>Heelalige Railway Station</t>
+  </si>
+  <si>
+    <t>Upcoming Namma Metro Yellow Line (Bommasandra Station - Approx. 10 - 12 km)</t>
+  </si>
+  <si>
+    <t>Immediate access to Panathur Road</t>
+  </si>
+  <si>
+    <t>45 - 60 km</t>
   </si>
   <si>
     <t>Heelalige</t>
   </si>
   <si>
-    <t>Upcoming Namma Metro Yellow Line</t>
-  </si>
-  <si>
-    <t>Immediate access</t>
-  </si>
-  <si>
-    <t>Metro Phase 2A/2B</t>
-  </si>
-  <si>
-    <t>0 km</t>
-  </si>
-  <si>
-    <t>25 mins</t>
-  </si>
-  <si>
-    <t>Yelahanka Junction</t>
-  </si>
-  <si>
-    <t>Upcoming Nagawara</t>
-  </si>
-  <si>
-    <t>25-30 km</t>
-  </si>
-  <si>
-    <t>KR Puram</t>
-  </si>
-  <si>
-    <t>KR Puram Metro</t>
-  </si>
-  <si>
-    <t>27-32 km</t>
-  </si>
-  <si>
-    <t>30-35 km</t>
-  </si>
-  <si>
-    <t>Whitefield</t>
-  </si>
-  <si>
-    <t>Whitefield Metro</t>
+    <t>Metro Phase 2A/2B (proposed)</t>
+  </si>
+  <si>
+    <t>0 km (Located directly on Thanisandra Main Road)</t>
+  </si>
+  <si>
+    <t>~25 mins (via New Airport Road)</t>
+  </si>
+  <si>
+    <t>~15 mins (Yelahanka Junction)</t>
+  </si>
+  <si>
+    <t>~10 mins (Upcoming Nagawara/Hebbal Metro - Blue/Pink Line)</t>
+  </si>
+  <si>
+    <t>0 km Located directly on main road</t>
+  </si>
+  <si>
+    <t>~25 - 30 km (Kempegowda International Airport - BLR)</t>
+  </si>
+  <si>
+    <t>KR Puram Railway Station (~10 - 12 km)</t>
+  </si>
+  <si>
+    <t>KR Puram Metro (~10 - 12 km)</t>
+  </si>
+  <si>
+    <t>0 km Located directly on Old Madras Road (OMR)</t>
+  </si>
+  <si>
+    <t>~27 - 32 km (Kempegowda International Airport - BLR | 45 - 60 mins)</t>
+  </si>
+  <si>
+    <t>KR Puram Railway Station (~9 - 11 km | 20 - 30 mins)</t>
+  </si>
+  <si>
+    <t>KR Puram Metro (~9 - 11 km | 20 - 25 mins)</t>
+  </si>
+  <si>
+    <t>0 km Located directly on Whitefield-Hoskote Road (Hope Farm Soukya Road belt)</t>
+  </si>
+  <si>
+    <t>~30 - 35 km (Kempegowda International Airport - BLR | ~40 - 50 mins)</t>
+  </si>
+  <si>
+    <t>Whitefield Railway Station (~10 - 12 km | ~20 - 25 mins)</t>
+  </si>
+  <si>
+    <t>Whitefield (Kadugodi) Metro (~10 - 12 km | ~20 - 25 mins)</t>
+  </si>
+  <si>
+    <t>0 km Located directly on Old Madras Road (near Hoskote Toll Gate)</t>
+  </si>
+  <si>
+    <t>~30 - 35 km (Kempegowda International Airport - BLR | 40 - 50 mins)</t>
+  </si>
+  <si>
+    <t>KR Puram Railway Station (~10 - 12 km | 20 - 30 mins)</t>
+  </si>
+  <si>
+    <t>Whitefield (Kadugodi) Metro (~15 - 18 km | 30 - 40 mins)</t>
   </si>
   <si>
     <t>customer_name</t>
@@ -1345,61 +1564,88 @@
       <c r="C2" t="s">
         <v>35</v>
       </c>
+      <c r="D2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" t="s">
+        <v>36</v>
+      </c>
       <c r="H2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I2">
         <v>2</v>
       </c>
       <c r="J2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="S2" t="s">
-        <v>39</v>
+        <v>40</v>
+      </c>
+      <c r="T2" t="s">
+        <v>41</v>
       </c>
       <c r="U2">
         <v>64</v>
       </c>
+      <c r="V2" t="s">
+        <v>42</v>
+      </c>
       <c r="W2">
         <v>10200000</v>
       </c>
       <c r="X2">
         <v>30600000</v>
       </c>
+      <c r="AB2" t="s">
+        <v>43</v>
+      </c>
       <c r="AG2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
         <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>46</v>
+      </c>
+      <c r="D3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" t="s">
+        <v>36</v>
       </c>
       <c r="H3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="I3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="K3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="S3" t="s">
-        <v>45</v>
+        <v>49</v>
+      </c>
+      <c r="T3" t="s">
+        <v>50</v>
       </c>
       <c r="U3">
-        <v>1875</v>
+        <v>1</v>
+      </c>
+      <c r="V3" t="s">
+        <v>51</v>
       </c>
       <c r="W3">
         <v>12000000</v>
@@ -1407,189 +1653,255 @@
       <c r="X3">
         <v>36000000</v>
       </c>
+      <c r="AB3" t="s">
+        <v>52</v>
+      </c>
       <c r="AG3" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B4" t="s">
         <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>48</v>
+        <v>55</v>
+      </c>
+      <c r="D4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
       </c>
       <c r="H4" t="s">
-        <v>49</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
+        <v>56</v>
       </c>
       <c r="J4" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="K4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="S4" t="s">
-        <v>51</v>
+        <v>58</v>
+      </c>
+      <c r="T4" t="s">
+        <v>59</v>
       </c>
       <c r="U4">
         <v>558</v>
       </c>
+      <c r="V4" t="s">
+        <v>51</v>
+      </c>
       <c r="W4">
         <v>12000000</v>
       </c>
       <c r="X4">
         <v>36000000</v>
       </c>
+      <c r="AB4" t="s">
+        <v>60</v>
+      </c>
       <c r="AG4" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="B5" t="s">
         <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>54</v>
+        <v>63</v>
+      </c>
+      <c r="D5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E5" t="s">
+        <v>36</v>
       </c>
       <c r="H5" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="I5">
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="K5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="S5" t="s">
-        <v>57</v>
+        <v>66</v>
+      </c>
+      <c r="T5" t="s">
+        <v>67</v>
       </c>
       <c r="U5">
         <v>1750</v>
       </c>
+      <c r="V5" t="s">
+        <v>68</v>
+      </c>
       <c r="W5">
         <v>11761000</v>
       </c>
       <c r="X5">
         <v>35283000</v>
       </c>
+      <c r="AB5" t="s">
+        <v>69</v>
+      </c>
       <c r="AG5" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="B6" t="s">
         <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>72</v>
+      </c>
+      <c r="D6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E6" t="s">
+        <v>36</v>
       </c>
       <c r="H6" t="s">
-        <v>61</v>
-      </c>
-      <c r="I6">
-        <v>1</v>
+        <v>73</v>
       </c>
       <c r="J6" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="K6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="S6" t="s">
-        <v>63</v>
+        <v>75</v>
+      </c>
+      <c r="T6" t="s">
+        <v>76</v>
       </c>
       <c r="U6">
         <v>394</v>
       </c>
+      <c r="V6" t="s">
+        <v>77</v>
+      </c>
       <c r="W6">
         <v>9800000</v>
       </c>
       <c r="X6">
         <v>29400000</v>
       </c>
+      <c r="AB6" t="s">
+        <v>78</v>
+      </c>
       <c r="AG6" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="B7" t="s">
         <v>34</v>
       </c>
       <c r="C7" t="s">
-        <v>66</v>
+        <v>81</v>
+      </c>
+      <c r="D7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E7" t="s">
+        <v>36</v>
       </c>
       <c r="H7" t="s">
-        <v>67</v>
-      </c>
-      <c r="I7">
-        <v>1</v>
+        <v>82</v>
       </c>
       <c r="J7" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="K7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="S7" t="s">
-        <v>63</v>
+        <v>84</v>
+      </c>
+      <c r="T7" t="s">
+        <v>85</v>
       </c>
       <c r="U7">
         <v>1100</v>
       </c>
+      <c r="V7" t="s">
+        <v>86</v>
+      </c>
       <c r="W7">
         <v>12300000</v>
       </c>
       <c r="X7">
         <v>36900000</v>
       </c>
+      <c r="AB7" t="s">
+        <v>87</v>
+      </c>
       <c r="AG7" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="B8" t="s">
         <v>34</v>
       </c>
       <c r="C8" t="s">
-        <v>71</v>
+        <v>90</v>
+      </c>
+      <c r="D8" t="s">
+        <v>90</v>
+      </c>
+      <c r="E8" t="s">
+        <v>36</v>
       </c>
       <c r="H8" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="I8">
         <v>2</v>
       </c>
       <c r="J8" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="K8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="S8" t="s">
-        <v>74</v>
+        <v>93</v>
+      </c>
+      <c r="T8" t="s">
+        <v>94</v>
       </c>
       <c r="U8">
-        <v>1679</v>
+        <v>1</v>
+      </c>
+      <c r="V8" t="s">
+        <v>95</v>
       </c>
       <c r="W8">
         <v>10500000</v>
@@ -1597,37 +1909,49 @@
       <c r="X8">
         <v>31500000</v>
       </c>
+      <c r="AB8" t="s">
+        <v>96</v>
+      </c>
       <c r="AG8" t="s">
-        <v>75</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="B9" t="s">
         <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>77</v>
+        <v>99</v>
+      </c>
+      <c r="D9" t="s">
+        <v>99</v>
+      </c>
+      <c r="E9" t="s">
+        <v>36</v>
       </c>
       <c r="H9" t="s">
-        <v>78</v>
-      </c>
-      <c r="I9">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="J9" t="s">
-        <v>79</v>
+        <v>101</v>
       </c>
       <c r="K9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="S9" t="s">
-        <v>74</v>
+        <v>102</v>
+      </c>
+      <c r="T9" t="s">
+        <v>103</v>
       </c>
       <c r="U9">
-        <v>3484</v>
+        <v>3</v>
+      </c>
+      <c r="V9" t="s">
+        <v>104</v>
       </c>
       <c r="W9">
         <v>11500000</v>
@@ -1635,8 +1959,11 @@
       <c r="X9">
         <v>34500000</v>
       </c>
+      <c r="AB9" t="s">
+        <v>105</v>
+      </c>
       <c r="AG9" t="s">
-        <v>80</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -1655,19 +1982,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>241</v>
+        <v>303</v>
       </c>
       <c r="C1" t="s">
-        <v>242</v>
+        <v>304</v>
       </c>
       <c r="D1" t="s">
-        <v>243</v>
+        <v>305</v>
       </c>
       <c r="E1" t="s">
-        <v>244</v>
+        <v>306</v>
       </c>
       <c r="F1" t="s">
-        <v>245</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1675,135 +2002,135 @@
         <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>246</v>
+        <v>308</v>
       </c>
       <c r="C2" t="s">
-        <v>247</v>
+        <v>309</v>
       </c>
       <c r="D2" t="s">
-        <v>248</v>
+        <v>310</v>
       </c>
       <c r="E2" t="s">
-        <v>249</v>
+        <v>311</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
-        <v>250</v>
+        <v>312</v>
       </c>
       <c r="C3" t="s">
-        <v>247</v>
+        <v>313</v>
       </c>
       <c r="D3" t="s">
-        <v>248</v>
+        <v>314</v>
       </c>
       <c r="E3" t="s">
-        <v>251</v>
+        <v>315</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B4" t="s">
-        <v>252</v>
+        <v>316</v>
       </c>
       <c r="C4" t="s">
-        <v>253</v>
+        <v>317</v>
       </c>
       <c r="D4" t="s">
-        <v>254</v>
+        <v>318</v>
       </c>
       <c r="E4" t="s">
-        <v>255</v>
+        <v>319</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="B5" t="s">
-        <v>252</v>
+        <v>320</v>
       </c>
       <c r="C5" t="s">
-        <v>256</v>
+        <v>321</v>
       </c>
       <c r="D5" t="s">
-        <v>257</v>
+        <v>322</v>
       </c>
       <c r="E5" t="s">
-        <v>258</v>
+        <v>323</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="B6" t="s">
-        <v>252</v>
+        <v>324</v>
       </c>
       <c r="C6" t="s">
-        <v>259</v>
+        <v>325</v>
       </c>
       <c r="D6" t="s">
-        <v>257</v>
+        <v>326</v>
       </c>
       <c r="E6" t="s">
-        <v>258</v>
+        <v>327</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="B7" t="s">
-        <v>252</v>
+        <v>328</v>
       </c>
       <c r="C7" t="s">
-        <v>260</v>
+        <v>329</v>
       </c>
       <c r="D7" t="s">
-        <v>261</v>
+        <v>330</v>
       </c>
       <c r="E7" t="s">
-        <v>262</v>
+        <v>331</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="B8" t="s">
-        <v>252</v>
+        <v>320</v>
       </c>
       <c r="C8" t="s">
-        <v>256</v>
+        <v>321</v>
       </c>
       <c r="D8" t="s">
-        <v>257</v>
+        <v>322</v>
       </c>
       <c r="E8" t="s">
-        <v>258</v>
+        <v>323</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="B9" t="s">
-        <v>252</v>
+        <v>332</v>
       </c>
       <c r="C9" t="s">
-        <v>260</v>
+        <v>333</v>
       </c>
       <c r="D9" t="s">
-        <v>257</v>
+        <v>334</v>
       </c>
       <c r="E9" t="s">
-        <v>262</v>
+        <v>335</v>
       </c>
     </row>
   </sheetData>
@@ -1822,22 +2149,22 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>263</v>
+        <v>336</v>
       </c>
       <c r="C1" t="s">
-        <v>264</v>
+        <v>337</v>
       </c>
       <c r="D1" t="s">
-        <v>265</v>
+        <v>338</v>
       </c>
       <c r="E1" t="s">
-        <v>266</v>
+        <v>339</v>
       </c>
       <c r="F1" t="s">
-        <v>152</v>
+        <v>201</v>
       </c>
       <c r="G1" t="s">
-        <v>267</v>
+        <v>340</v>
       </c>
     </row>
   </sheetData>
@@ -1856,19 +2183,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>81</v>
+        <v>107</v>
       </c>
       <c r="C1" t="s">
-        <v>268</v>
+        <v>341</v>
       </c>
       <c r="D1" t="s">
-        <v>269</v>
+        <v>342</v>
       </c>
       <c r="E1" t="s">
-        <v>152</v>
+        <v>201</v>
       </c>
       <c r="F1" t="s">
-        <v>270</v>
+        <v>343</v>
       </c>
     </row>
   </sheetData>
@@ -1884,16 +2211,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>268</v>
+        <v>341</v>
       </c>
       <c r="B1" t="s">
-        <v>271</v>
+        <v>344</v>
       </c>
       <c r="C1" t="s">
-        <v>272</v>
+        <v>345</v>
       </c>
       <c r="D1" t="s">
-        <v>273</v>
+        <v>346</v>
       </c>
     </row>
   </sheetData>
@@ -1909,16 +2236,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>274</v>
+        <v>347</v>
       </c>
       <c r="B1" t="s">
-        <v>275</v>
+        <v>348</v>
       </c>
       <c r="C1" t="s">
-        <v>152</v>
+        <v>201</v>
       </c>
       <c r="D1" t="s">
-        <v>276</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -1937,98 +2264,215 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>81</v>
+        <v>107</v>
       </c>
       <c r="C1" t="s">
-        <v>82</v>
+        <v>108</v>
       </c>
       <c r="D1" t="s">
-        <v>83</v>
+        <v>109</v>
       </c>
       <c r="E1" t="s">
-        <v>84</v>
+        <v>110</v>
       </c>
       <c r="F1" t="s">
-        <v>85</v>
+        <v>111</v>
       </c>
       <c r="G1" t="s">
-        <v>86</v>
+        <v>112</v>
       </c>
       <c r="H1" t="s">
-        <v>87</v>
+        <v>113</v>
       </c>
       <c r="I1" t="s">
-        <v>88</v>
+        <v>114</v>
       </c>
       <c r="J1" t="s">
-        <v>89</v>
+        <v>115</v>
       </c>
       <c r="K1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+      <c r="G2" t="s">
+        <v>118</v>
+      </c>
+      <c r="H2" t="s">
+        <v>119</v>
+      </c>
+      <c r="J2" t="s">
+        <v>119</v>
+      </c>
+      <c r="K2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+      <c r="G3" t="s">
+        <v>122</v>
+      </c>
+      <c r="H3" t="s">
+        <v>123</v>
+      </c>
+      <c r="I3">
+        <v>28</v>
+      </c>
+      <c r="J3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B4" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+      <c r="G4" t="s">
+        <v>127</v>
+      </c>
+      <c r="H4" t="s">
+        <v>128</v>
+      </c>
+      <c r="I4">
+        <v>30</v>
+      </c>
+      <c r="J4" t="s">
+        <v>129</v>
+      </c>
+      <c r="K4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="B5" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>131</v>
+      </c>
+      <c r="G5" t="s">
+        <v>132</v>
+      </c>
+      <c r="H5" t="s">
+        <v>133</v>
+      </c>
+      <c r="I5">
+        <v>35</v>
+      </c>
+      <c r="J5" t="s">
+        <v>134</v>
+      </c>
+      <c r="K5" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="B6" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+      <c r="G6" t="s">
+        <v>137</v>
+      </c>
+      <c r="H6" t="s">
+        <v>138</v>
+      </c>
+      <c r="I6">
+        <v>30</v>
+      </c>
+      <c r="J6" t="s">
+        <v>139</v>
+      </c>
+      <c r="K6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="B7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+      <c r="G7" t="s">
+        <v>141</v>
+      </c>
+      <c r="H7" t="s">
+        <v>142</v>
+      </c>
+      <c r="I7">
+        <v>30</v>
+      </c>
+      <c r="J7" t="s">
+        <v>143</v>
+      </c>
+      <c r="K7" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="B8" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+      <c r="G8" t="s">
+        <v>146</v>
+      </c>
+      <c r="H8" t="s">
+        <v>147</v>
+      </c>
+      <c r="I8">
+        <v>30</v>
+      </c>
+      <c r="J8" t="s">
+        <v>148</v>
+      </c>
+      <c r="K8" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="B9" t="s">
-        <v>92</v>
+        <v>121</v>
+      </c>
+      <c r="G9" t="s">
+        <v>150</v>
+      </c>
+      <c r="H9" t="s">
+        <v>151</v>
+      </c>
+      <c r="I9">
+        <v>35</v>
+      </c>
+      <c r="J9" t="s">
+        <v>152</v>
+      </c>
+      <c r="K9" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -2047,34 +2491,34 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>98</v>
+        <v>153</v>
       </c>
       <c r="C1" t="s">
-        <v>99</v>
+        <v>154</v>
       </c>
       <c r="D1" t="s">
-        <v>100</v>
+        <v>155</v>
       </c>
       <c r="E1" t="s">
-        <v>101</v>
+        <v>156</v>
       </c>
       <c r="F1" t="s">
-        <v>102</v>
+        <v>157</v>
       </c>
       <c r="G1" t="s">
-        <v>103</v>
+        <v>158</v>
       </c>
       <c r="H1" t="s">
-        <v>104</v>
+        <v>159</v>
       </c>
       <c r="I1" t="s">
-        <v>105</v>
+        <v>160</v>
       </c>
       <c r="J1" t="s">
-        <v>106</v>
+        <v>161</v>
       </c>
       <c r="K1" t="s">
-        <v>107</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -2082,135 +2526,159 @@
         <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>108</v>
+        <v>163</v>
       </c>
       <c r="C2" t="s">
-        <v>109</v>
+        <v>164</v>
       </c>
       <c r="D2" t="s">
-        <v>110</v>
+        <v>165</v>
+      </c>
+      <c r="E2" t="s">
+        <v>165</v>
       </c>
       <c r="G2" t="s">
-        <v>111</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
-        <v>112</v>
+        <v>167</v>
       </c>
       <c r="C3" t="s">
-        <v>113</v>
+        <v>164</v>
       </c>
       <c r="D3" t="s">
-        <v>114</v>
+        <v>168</v>
+      </c>
+      <c r="E3" t="s">
+        <v>168</v>
       </c>
       <c r="G3" t="s">
-        <v>115</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B4" t="s">
-        <v>116</v>
+        <v>170</v>
       </c>
       <c r="C4" t="s">
-        <v>117</v>
+        <v>164</v>
       </c>
       <c r="D4" t="s">
-        <v>118</v>
+        <v>171</v>
+      </c>
+      <c r="E4" t="s">
+        <v>171</v>
       </c>
       <c r="G4" t="s">
-        <v>119</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="B5" t="s">
-        <v>120</v>
+        <v>173</v>
       </c>
       <c r="C5" t="s">
-        <v>121</v>
+        <v>164</v>
       </c>
       <c r="D5" t="s">
-        <v>122</v>
+        <v>174</v>
+      </c>
+      <c r="E5" t="s">
+        <v>174</v>
       </c>
       <c r="G5" t="s">
-        <v>123</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="B6" t="s">
-        <v>124</v>
+        <v>176</v>
       </c>
       <c r="C6" t="s">
-        <v>125</v>
+        <v>164</v>
       </c>
       <c r="D6" t="s">
-        <v>126</v>
+        <v>177</v>
+      </c>
+      <c r="E6" t="s">
+        <v>177</v>
       </c>
       <c r="G6" t="s">
-        <v>127</v>
+        <v>178</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="B7" t="s">
-        <v>128</v>
+        <v>179</v>
       </c>
       <c r="C7" t="s">
-        <v>129</v>
+        <v>164</v>
       </c>
       <c r="D7" t="s">
-        <v>73</v>
+        <v>180</v>
+      </c>
+      <c r="E7" t="s">
+        <v>180</v>
       </c>
       <c r="G7" t="s">
-        <v>130</v>
+        <v>181</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="B8" t="s">
-        <v>131</v>
+        <v>182</v>
       </c>
       <c r="C8" t="s">
-        <v>132</v>
+        <v>164</v>
       </c>
       <c r="D8" t="s">
-        <v>133</v>
+        <v>183</v>
+      </c>
+      <c r="E8" t="s">
+        <v>183</v>
       </c>
       <c r="G8" t="s">
-        <v>134</v>
+        <v>184</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="B9" t="s">
-        <v>135</v>
+        <v>185</v>
       </c>
       <c r="C9" t="s">
-        <v>136</v>
+        <v>164</v>
       </c>
       <c r="D9" t="s">
-        <v>137</v>
+        <v>186</v>
+      </c>
+      <c r="E9" t="s">
+        <v>186</v>
       </c>
       <c r="G9" t="s">
-        <v>138</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -2229,46 +2697,46 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>139</v>
+        <v>188</v>
       </c>
       <c r="C1" t="s">
-        <v>140</v>
+        <v>189</v>
       </c>
       <c r="D1" t="s">
-        <v>141</v>
+        <v>190</v>
       </c>
       <c r="E1" t="s">
-        <v>142</v>
+        <v>191</v>
       </c>
       <c r="F1" t="s">
-        <v>143</v>
+        <v>192</v>
       </c>
       <c r="G1" t="s">
-        <v>144</v>
+        <v>193</v>
       </c>
       <c r="H1" t="s">
-        <v>145</v>
+        <v>194</v>
       </c>
       <c r="I1" t="s">
-        <v>146</v>
+        <v>195</v>
       </c>
       <c r="J1" t="s">
-        <v>147</v>
+        <v>196</v>
       </c>
       <c r="K1" t="s">
-        <v>148</v>
+        <v>197</v>
       </c>
       <c r="L1" t="s">
-        <v>149</v>
+        <v>198</v>
       </c>
       <c r="M1" t="s">
-        <v>150</v>
+        <v>199</v>
       </c>
       <c r="N1" t="s">
-        <v>151</v>
+        <v>200</v>
       </c>
       <c r="O1" t="s">
-        <v>152</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -2276,10 +2744,10 @@
         <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>153</v>
+        <v>202</v>
       </c>
       <c r="E2" t="s">
-        <v>154</v>
+        <v>203</v>
       </c>
       <c r="G2">
         <v>3923</v>
@@ -2294,7 +2762,7 @@
         <v>40014600</v>
       </c>
       <c r="O2" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -2302,10 +2770,10 @@
         <v>33</v>
       </c>
       <c r="B3" t="s">
-        <v>156</v>
+        <v>205</v>
       </c>
       <c r="E3" t="s">
-        <v>154</v>
+        <v>203</v>
       </c>
       <c r="G3">
         <v>3959</v>
@@ -2320,7 +2788,7 @@
         <v>40381800</v>
       </c>
       <c r="O3" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -2328,10 +2796,10 @@
         <v>33</v>
       </c>
       <c r="B4" t="s">
-        <v>157</v>
+        <v>206</v>
       </c>
       <c r="E4" t="s">
-        <v>154</v>
+        <v>203</v>
       </c>
       <c r="G4">
         <v>4894</v>
@@ -2346,7 +2814,7 @@
         <v>49918800</v>
       </c>
       <c r="O4" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -2354,10 +2822,10 @@
         <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>158</v>
+        <v>207</v>
       </c>
       <c r="E5" t="s">
-        <v>159</v>
+        <v>208</v>
       </c>
       <c r="G5">
         <v>4836</v>
@@ -2372,18 +2840,18 @@
         <v>49327200</v>
       </c>
       <c r="O5" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>160</v>
+        <v>209</v>
       </c>
       <c r="E6" t="s">
-        <v>161</v>
+        <v>210</v>
       </c>
       <c r="G6">
         <v>660</v>
@@ -2398,18 +2866,18 @@
         <v>7920000</v>
       </c>
       <c r="O6" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>162</v>
+        <v>211</v>
       </c>
       <c r="E7" t="s">
-        <v>163</v>
+        <v>212</v>
       </c>
       <c r="G7">
         <v>1611</v>
@@ -2421,18 +2889,18 @@
         <v>19332000</v>
       </c>
       <c r="O7" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>164</v>
+        <v>213</v>
       </c>
       <c r="E8" t="s">
-        <v>165</v>
+        <v>214</v>
       </c>
       <c r="G8">
         <v>2333</v>
@@ -2444,18 +2912,18 @@
         <v>27996000</v>
       </c>
       <c r="O8" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B9" t="s">
-        <v>166</v>
+        <v>215</v>
       </c>
       <c r="E9" t="s">
-        <v>167</v>
+        <v>216</v>
       </c>
       <c r="G9">
         <v>1242</v>
@@ -2467,18 +2935,18 @@
         <v>14904000</v>
       </c>
       <c r="O9" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B10" t="s">
-        <v>168</v>
+        <v>217</v>
       </c>
       <c r="E10" t="s">
-        <v>169</v>
+        <v>212</v>
       </c>
       <c r="G10">
         <v>1887</v>
@@ -2490,18 +2958,18 @@
         <v>22644000</v>
       </c>
       <c r="O10" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B11" t="s">
-        <v>170</v>
+        <v>218</v>
       </c>
       <c r="E11" t="s">
-        <v>171</v>
+        <v>219</v>
       </c>
       <c r="G11">
         <v>2191</v>
@@ -2513,18 +2981,18 @@
         <v>26292000</v>
       </c>
       <c r="O11" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="B12" t="s">
-        <v>172</v>
+        <v>220</v>
       </c>
       <c r="E12" t="s">
-        <v>161</v>
+        <v>210</v>
       </c>
       <c r="G12">
         <v>715</v>
@@ -2536,18 +3004,18 @@
         <v>8409115</v>
       </c>
       <c r="O12" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="B13" t="s">
-        <v>173</v>
+        <v>221</v>
       </c>
       <c r="E13" t="s">
-        <v>167</v>
+        <v>216</v>
       </c>
       <c r="G13">
         <v>1111</v>
@@ -2559,18 +3027,18 @@
         <v>13066471</v>
       </c>
       <c r="O13" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="B14" t="s">
-        <v>174</v>
+        <v>222</v>
       </c>
       <c r="E14" t="s">
-        <v>163</v>
+        <v>212</v>
       </c>
       <c r="G14">
         <v>1720</v>
@@ -2582,18 +3050,18 @@
         <v>20228920</v>
       </c>
       <c r="O14" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="B15" t="s">
-        <v>175</v>
+        <v>223</v>
       </c>
       <c r="E15" t="s">
-        <v>163</v>
+        <v>212</v>
       </c>
       <c r="G15">
         <v>1389</v>
@@ -2605,18 +3073,18 @@
         <v>13612200</v>
       </c>
       <c r="O15" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="B16" t="s">
-        <v>176</v>
+        <v>224</v>
       </c>
       <c r="E16" t="s">
-        <v>167</v>
+        <v>216</v>
       </c>
       <c r="G16">
         <v>1063</v>
@@ -2628,18 +3096,18 @@
         <v>13074900</v>
       </c>
       <c r="O16" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="B17" t="s">
-        <v>177</v>
+        <v>225</v>
       </c>
       <c r="E17" t="s">
-        <v>163</v>
+        <v>212</v>
       </c>
       <c r="G17">
         <v>1510</v>
@@ -2651,18 +3119,18 @@
         <v>18573000</v>
       </c>
       <c r="O17" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="B18" t="s">
-        <v>178</v>
+        <v>226</v>
       </c>
       <c r="E18" t="s">
-        <v>161</v>
+        <v>210</v>
       </c>
       <c r="G18">
         <v>753</v>
@@ -2674,18 +3142,18 @@
         <v>7906500</v>
       </c>
       <c r="O18" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="B19" t="s">
-        <v>179</v>
+        <v>227</v>
       </c>
       <c r="E19" t="s">
-        <v>167</v>
+        <v>216</v>
       </c>
       <c r="G19">
         <v>1268</v>
@@ -2697,18 +3165,18 @@
         <v>13314000</v>
       </c>
       <c r="O19" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="B20" t="s">
-        <v>180</v>
+        <v>228</v>
       </c>
       <c r="E20" t="s">
-        <v>163</v>
+        <v>212</v>
       </c>
       <c r="G20">
         <v>1733</v>
@@ -2720,18 +3188,18 @@
         <v>18196500</v>
       </c>
       <c r="O20" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="B21" t="s">
-        <v>181</v>
+        <v>229</v>
       </c>
       <c r="E21" t="s">
-        <v>182</v>
+        <v>230</v>
       </c>
       <c r="G21">
         <v>3336</v>
@@ -2743,18 +3211,18 @@
         <v>35028000</v>
       </c>
       <c r="O21" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="B22" t="s">
-        <v>183</v>
+        <v>231</v>
       </c>
       <c r="E22" t="s">
-        <v>161</v>
+        <v>210</v>
       </c>
       <c r="G22">
         <v>734</v>
@@ -2766,18 +3234,18 @@
         <v>8441000</v>
       </c>
       <c r="O22" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="B23" t="s">
-        <v>184</v>
+        <v>232</v>
       </c>
       <c r="E23" t="s">
-        <v>167</v>
+        <v>216</v>
       </c>
       <c r="G23">
         <v>1063</v>
@@ -2789,18 +3257,18 @@
         <v>12224500</v>
       </c>
       <c r="O23" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="B24" t="s">
-        <v>185</v>
+        <v>233</v>
       </c>
       <c r="E24" t="s">
-        <v>163</v>
+        <v>212</v>
       </c>
       <c r="G24">
         <v>1510</v>
@@ -2812,18 +3280,18 @@
         <v>17365000</v>
       </c>
       <c r="O24" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="B25" t="s">
-        <v>186</v>
+        <v>234</v>
       </c>
       <c r="E25" t="s">
-        <v>165</v>
+        <v>214</v>
       </c>
       <c r="G25">
         <v>2096</v>
@@ -2835,7 +3303,7 @@
         <v>24104000</v>
       </c>
       <c r="O25" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -2854,88 +3322,88 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>187</v>
+        <v>235</v>
       </c>
       <c r="C1" t="s">
-        <v>188</v>
+        <v>236</v>
       </c>
       <c r="D1" t="s">
-        <v>189</v>
+        <v>237</v>
       </c>
       <c r="E1" t="s">
-        <v>190</v>
+        <v>238</v>
       </c>
       <c r="F1" t="s">
-        <v>191</v>
+        <v>239</v>
       </c>
       <c r="G1" t="s">
-        <v>192</v>
+        <v>240</v>
       </c>
       <c r="H1" t="s">
-        <v>193</v>
+        <v>241</v>
       </c>
       <c r="I1" t="s">
-        <v>194</v>
+        <v>242</v>
       </c>
       <c r="J1" t="s">
-        <v>195</v>
+        <v>243</v>
       </c>
       <c r="K1" t="s">
-        <v>196</v>
+        <v>244</v>
       </c>
       <c r="L1" t="s">
-        <v>197</v>
+        <v>245</v>
       </c>
       <c r="M1" t="s">
-        <v>198</v>
+        <v>246</v>
       </c>
       <c r="N1" t="s">
-        <v>199</v>
+        <v>247</v>
       </c>
       <c r="O1" t="s">
-        <v>200</v>
+        <v>248</v>
       </c>
       <c r="P1" t="s">
-        <v>201</v>
+        <v>249</v>
       </c>
       <c r="Q1" t="s">
-        <v>202</v>
+        <v>250</v>
       </c>
       <c r="R1" t="s">
-        <v>203</v>
+        <v>251</v>
       </c>
       <c r="S1" t="s">
-        <v>204</v>
+        <v>252</v>
       </c>
       <c r="T1" t="s">
-        <v>205</v>
+        <v>253</v>
       </c>
       <c r="U1" t="s">
-        <v>206</v>
+        <v>254</v>
       </c>
       <c r="V1" t="s">
-        <v>207</v>
+        <v>255</v>
       </c>
       <c r="W1" t="s">
-        <v>208</v>
+        <v>256</v>
       </c>
       <c r="X1" t="s">
-        <v>209</v>
+        <v>257</v>
       </c>
       <c r="Y1" t="s">
-        <v>210</v>
+        <v>258</v>
       </c>
       <c r="Z1" t="s">
-        <v>211</v>
+        <v>259</v>
       </c>
       <c r="AA1" t="s">
-        <v>212</v>
+        <v>260</v>
       </c>
       <c r="AB1" t="s">
-        <v>213</v>
+        <v>261</v>
       </c>
       <c r="AC1" t="s">
-        <v>214</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2" spans="1:29" x14ac:dyDescent="0.25">
@@ -2952,15 +3420,15 @@
         <v>1</v>
       </c>
       <c r="G2" t="s">
-        <v>215</v>
-      </c>
-      <c r="AC2">
-        <v>60</v>
+        <v>263</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B3">
         <v>19</v>
@@ -2972,15 +3440,15 @@
         <v>8</v>
       </c>
       <c r="G3" t="s">
-        <v>216</v>
-      </c>
-      <c r="AC3">
-        <v>78</v>
+        <v>265</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B4">
         <v>10</v>
@@ -2992,18 +3460,18 @@
         <v>5</v>
       </c>
       <c r="G4" t="s">
-        <v>217</v>
-      </c>
-      <c r="AC4">
-        <v>76</v>
+        <v>267</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="C5">
         <v>43</v>
@@ -3012,15 +3480,15 @@
         <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>218</v>
-      </c>
-      <c r="AC5">
-        <v>81</v>
+        <v>269</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="B6">
         <v>2</v>
@@ -3032,15 +3500,15 @@
         <v>8</v>
       </c>
       <c r="G6" t="s">
-        <v>219</v>
-      </c>
-      <c r="AC6">
-        <v>60</v>
+        <v>271</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="B7">
         <v>5</v>
@@ -3052,18 +3520,18 @@
         <v>8</v>
       </c>
       <c r="G7" t="s">
-        <v>220</v>
-      </c>
-      <c r="AC7">
-        <v>80</v>
+        <v>272</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="B8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C8">
         <v>31</v>
@@ -3072,15 +3540,15 @@
         <v>8</v>
       </c>
       <c r="G8" t="s">
-        <v>221</v>
-      </c>
-      <c r="AC8">
-        <v>80</v>
+        <v>274</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="B9">
         <v>14</v>
@@ -3092,10 +3560,10 @@
         <v>8</v>
       </c>
       <c r="G9" t="s">
-        <v>222</v>
-      </c>
-      <c r="AC9">
-        <v>80</v>
+        <v>275</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>273</v>
       </c>
     </row>
   </sheetData>
@@ -3114,16 +3582,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>223</v>
+        <v>276</v>
       </c>
       <c r="C1" t="s">
-        <v>81</v>
+        <v>107</v>
       </c>
       <c r="D1" t="s">
-        <v>86</v>
+        <v>112</v>
       </c>
       <c r="E1" t="s">
-        <v>224</v>
+        <v>277</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -3131,111 +3599,111 @@
         <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>225</v>
+        <v>278</v>
       </c>
       <c r="C2" t="s">
-        <v>226</v>
+        <v>279</v>
       </c>
       <c r="E2" t="s">
-        <v>227</v>
+        <v>280</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
-        <v>225</v>
+        <v>278</v>
       </c>
       <c r="C3" t="s">
-        <v>226</v>
+        <v>279</v>
       </c>
       <c r="E3" t="s">
-        <v>228</v>
+        <v>281</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B4" t="s">
-        <v>225</v>
+        <v>278</v>
       </c>
       <c r="C4" t="s">
-        <v>226</v>
+        <v>279</v>
       </c>
       <c r="E4" t="s">
-        <v>229</v>
+        <v>282</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="B5" t="s">
-        <v>225</v>
+        <v>278</v>
       </c>
       <c r="C5" t="s">
-        <v>226</v>
+        <v>279</v>
       </c>
       <c r="E5" t="s">
-        <v>230</v>
+        <v>283</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="B6" t="s">
-        <v>225</v>
+        <v>278</v>
       </c>
       <c r="C6" t="s">
-        <v>226</v>
+        <v>279</v>
       </c>
       <c r="E6" t="s">
-        <v>231</v>
+        <v>284</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="B7" t="s">
-        <v>225</v>
+        <v>278</v>
       </c>
       <c r="C7" t="s">
-        <v>226</v>
+        <v>279</v>
       </c>
       <c r="E7" t="s">
-        <v>232</v>
+        <v>285</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="B8" t="s">
-        <v>225</v>
+        <v>278</v>
       </c>
       <c r="C8" t="s">
-        <v>226</v>
+        <v>279</v>
       </c>
       <c r="E8" t="s">
-        <v>233</v>
+        <v>286</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="B9" t="s">
-        <v>225</v>
+        <v>278</v>
       </c>
       <c r="C9" t="s">
-        <v>226</v>
+        <v>279</v>
       </c>
       <c r="E9" t="s">
-        <v>234</v>
+        <v>287</v>
       </c>
     </row>
   </sheetData>
@@ -3246,7 +3714,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3254,16 +3722,104 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>223</v>
+        <v>276</v>
       </c>
       <c r="C1" t="s">
-        <v>81</v>
+        <v>107</v>
       </c>
       <c r="D1" t="s">
-        <v>235</v>
+        <v>288</v>
       </c>
       <c r="E1" t="s">
-        <v>236</v>
+        <v>289</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>290</v>
+      </c>
+      <c r="C2" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" t="s">
+        <v>290</v>
+      </c>
+      <c r="C3" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" t="s">
+        <v>290</v>
+      </c>
+      <c r="C4" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" t="s">
+        <v>290</v>
+      </c>
+      <c r="C5" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" t="s">
+        <v>290</v>
+      </c>
+      <c r="C6" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>80</v>
+      </c>
+      <c r="B7" t="s">
+        <v>290</v>
+      </c>
+      <c r="C7" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>89</v>
+      </c>
+      <c r="B8" t="s">
+        <v>290</v>
+      </c>
+      <c r="C8" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B9" t="s">
+        <v>290</v>
+      </c>
+      <c r="C9" t="s">
+        <v>298</v>
       </c>
     </row>
   </sheetData>
@@ -3282,16 +3838,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>81</v>
+        <v>107</v>
       </c>
       <c r="C1" t="s">
-        <v>237</v>
+        <v>299</v>
       </c>
       <c r="D1" t="s">
-        <v>238</v>
+        <v>300</v>
       </c>
       <c r="E1" t="s">
-        <v>239</v>
+        <v>301</v>
       </c>
     </row>
   </sheetData>
@@ -3310,10 +3866,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>81</v>
+        <v>107</v>
       </c>
       <c r="C1" t="s">
-        <v>240</v>
+        <v>302</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Initial commit of geoestate
</commit_message>
<xml_diff>
--- a/Populated_Parity_Template.xlsx
+++ b/Populated_Parity_Template.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="349">
   <si>
     <t>project_name</t>
   </si>
@@ -126,9 +126,6 @@
   </si>
   <si>
     <t>Rainbow Mayfair</t>
-  </si>
-  <si>
-    <t>Admin</t>
   </si>
   <si>
     <t>General Location: Hullahalli, Bengaluru. Key Road Access: Off, Begur - Koppa Rd, Hullahalli. Detailed Address (Legal): SY NO 41/4, AND SY NO 43/1, HULLAHALLI VILLAGE, JIGANI HOBLI, Anekal. Nearby Landmark: Near BVM Global School.</t>
@@ -1558,41 +1555,38 @@
       <c r="A2" t="s">
         <v>33</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>34</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" t="s">
         <v>35</v>
       </c>
-      <c r="D2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="H2" t="s">
         <v>36</v>
-      </c>
-      <c r="H2" t="s">
-        <v>37</v>
       </c>
       <c r="I2">
         <v>2</v>
       </c>
       <c r="J2" t="s">
+        <v>37</v>
+      </c>
+      <c r="K2" t="s">
         <v>38</v>
       </c>
-      <c r="K2" t="s">
+      <c r="S2" t="s">
         <v>39</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>40</v>
-      </c>
-      <c r="T2" t="s">
-        <v>41</v>
       </c>
       <c r="U2">
         <v>64</v>
       </c>
       <c r="V2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="W2">
         <v>10200000</v>
@@ -1601,51 +1595,48 @@
         <v>30600000</v>
       </c>
       <c r="AB2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AG2" t="s">
         <v>43</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" t="s">
         <v>45</v>
       </c>
-      <c r="B3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H3" t="s">
         <v>46</v>
-      </c>
-      <c r="D3" t="s">
-        <v>46</v>
-      </c>
-      <c r="E3" t="s">
-        <v>36</v>
-      </c>
-      <c r="H3" t="s">
-        <v>47</v>
       </c>
       <c r="I3">
         <v>1</v>
       </c>
       <c r="J3" t="s">
+        <v>47</v>
+      </c>
+      <c r="K3" t="s">
+        <v>38</v>
+      </c>
+      <c r="S3" t="s">
         <v>48</v>
       </c>
-      <c r="K3" t="s">
-        <v>39</v>
-      </c>
-      <c r="S3" t="s">
+      <c r="T3" t="s">
         <v>49</v>
-      </c>
-      <c r="T3" t="s">
-        <v>50</v>
       </c>
       <c r="U3">
         <v>1</v>
       </c>
       <c r="V3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="W3">
         <v>12000000</v>
@@ -1654,48 +1645,45 @@
         <v>36000000</v>
       </c>
       <c r="AB3" t="s">
+        <v>51</v>
+      </c>
+      <c r="AG3" t="s">
         <v>52</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" t="s">
         <v>54</v>
       </c>
-      <c r="B4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H4" t="s">
         <v>55</v>
       </c>
-      <c r="D4" t="s">
-        <v>55</v>
-      </c>
-      <c r="E4" t="s">
-        <v>36</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="J4" t="s">
         <v>56</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
+        <v>38</v>
+      </c>
+      <c r="S4" t="s">
         <v>57</v>
       </c>
-      <c r="K4" t="s">
-        <v>39</v>
-      </c>
-      <c r="S4" t="s">
+      <c r="T4" t="s">
         <v>58</v>
-      </c>
-      <c r="T4" t="s">
-        <v>59</v>
       </c>
       <c r="U4">
         <v>558</v>
       </c>
       <c r="V4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="W4">
         <v>12000000</v>
@@ -1704,51 +1692,48 @@
         <v>36000000</v>
       </c>
       <c r="AB4" t="s">
+        <v>59</v>
+      </c>
+      <c r="AG4" t="s">
         <v>60</v>
-      </c>
-      <c r="AG4" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" t="s">
         <v>62</v>
       </c>
-      <c r="B5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
+        <v>62</v>
+      </c>
+      <c r="E5" t="s">
+        <v>35</v>
+      </c>
+      <c r="H5" t="s">
         <v>63</v>
-      </c>
-      <c r="D5" t="s">
-        <v>63</v>
-      </c>
-      <c r="E5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H5" t="s">
-        <v>64</v>
       </c>
       <c r="I5">
         <v>1</v>
       </c>
       <c r="J5" t="s">
+        <v>64</v>
+      </c>
+      <c r="K5" t="s">
+        <v>38</v>
+      </c>
+      <c r="S5" t="s">
         <v>65</v>
       </c>
-      <c r="K5" t="s">
-        <v>39</v>
-      </c>
-      <c r="S5" t="s">
+      <c r="T5" t="s">
         <v>66</v>
-      </c>
-      <c r="T5" t="s">
-        <v>67</v>
       </c>
       <c r="U5">
         <v>1750</v>
       </c>
       <c r="V5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="W5">
         <v>11761000</v>
@@ -1757,48 +1742,45 @@
         <v>35283000</v>
       </c>
       <c r="AB5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AG5" t="s">
         <v>69</v>
-      </c>
-      <c r="AG5" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6" t="s">
         <v>71</v>
       </c>
-      <c r="B6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
+        <v>71</v>
+      </c>
+      <c r="E6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H6" t="s">
         <v>72</v>
       </c>
-      <c r="D6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E6" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="J6" t="s">
         <v>73</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S6" t="s">
         <v>74</v>
       </c>
-      <c r="K6" t="s">
-        <v>39</v>
-      </c>
-      <c r="S6" t="s">
+      <c r="T6" t="s">
         <v>75</v>
-      </c>
-      <c r="T6" t="s">
-        <v>76</v>
       </c>
       <c r="U6">
         <v>394</v>
       </c>
       <c r="V6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="W6">
         <v>9800000</v>
@@ -1807,48 +1789,45 @@
         <v>29400000</v>
       </c>
       <c r="AB6" t="s">
+        <v>77</v>
+      </c>
+      <c r="AG6" t="s">
         <v>78</v>
-      </c>
-      <c r="AG6" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" t="s">
         <v>80</v>
       </c>
-      <c r="B7" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E7" t="s">
+        <v>35</v>
+      </c>
+      <c r="H7" t="s">
         <v>81</v>
       </c>
-      <c r="D7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E7" t="s">
-        <v>36</v>
-      </c>
-      <c r="H7" t="s">
+      <c r="J7" t="s">
         <v>82</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
+        <v>38</v>
+      </c>
+      <c r="S7" t="s">
         <v>83</v>
       </c>
-      <c r="K7" t="s">
-        <v>39</v>
-      </c>
-      <c r="S7" t="s">
+      <c r="T7" t="s">
         <v>84</v>
-      </c>
-      <c r="T7" t="s">
-        <v>85</v>
       </c>
       <c r="U7">
         <v>1100</v>
       </c>
       <c r="V7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="W7">
         <v>12300000</v>
@@ -1857,51 +1836,48 @@
         <v>36900000</v>
       </c>
       <c r="AB7" t="s">
+        <v>86</v>
+      </c>
+      <c r="AG7" t="s">
         <v>87</v>
-      </c>
-      <c r="AG7" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>88</v>
+      </c>
+      <c r="C8" t="s">
         <v>89</v>
       </c>
-      <c r="B8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
+        <v>89</v>
+      </c>
+      <c r="E8" t="s">
+        <v>35</v>
+      </c>
+      <c r="H8" t="s">
         <v>90</v>
-      </c>
-      <c r="D8" t="s">
-        <v>90</v>
-      </c>
-      <c r="E8" t="s">
-        <v>36</v>
-      </c>
-      <c r="H8" t="s">
-        <v>91</v>
       </c>
       <c r="I8">
         <v>2</v>
       </c>
       <c r="J8" t="s">
+        <v>91</v>
+      </c>
+      <c r="K8" t="s">
+        <v>38</v>
+      </c>
+      <c r="S8" t="s">
         <v>92</v>
       </c>
-      <c r="K8" t="s">
-        <v>39</v>
-      </c>
-      <c r="S8" t="s">
+      <c r="T8" t="s">
         <v>93</v>
-      </c>
-      <c r="T8" t="s">
-        <v>94</v>
       </c>
       <c r="U8">
         <v>1</v>
       </c>
       <c r="V8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="W8">
         <v>10500000</v>
@@ -1910,48 +1886,45 @@
         <v>31500000</v>
       </c>
       <c r="AB8" t="s">
+        <v>95</v>
+      </c>
+      <c r="AG8" t="s">
         <v>96</v>
-      </c>
-      <c r="AG8" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>97</v>
+      </c>
+      <c r="C9" t="s">
         <v>98</v>
       </c>
-      <c r="B9" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
+        <v>98</v>
+      </c>
+      <c r="E9" t="s">
+        <v>35</v>
+      </c>
+      <c r="H9" t="s">
         <v>99</v>
       </c>
-      <c r="D9" t="s">
-        <v>99</v>
-      </c>
-      <c r="E9" t="s">
-        <v>36</v>
-      </c>
-      <c r="H9" t="s">
+      <c r="J9" t="s">
         <v>100</v>
       </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
+        <v>38</v>
+      </c>
+      <c r="S9" t="s">
         <v>101</v>
       </c>
-      <c r="K9" t="s">
-        <v>39</v>
-      </c>
-      <c r="S9" t="s">
+      <c r="T9" t="s">
         <v>102</v>
-      </c>
-      <c r="T9" t="s">
-        <v>103</v>
       </c>
       <c r="U9">
         <v>3</v>
       </c>
       <c r="V9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="W9">
         <v>11500000</v>
@@ -1960,10 +1933,10 @@
         <v>34500000</v>
       </c>
       <c r="AB9" t="s">
+        <v>104</v>
+      </c>
+      <c r="AG9" t="s">
         <v>105</v>
-      </c>
-      <c r="AG9" t="s">
-        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -1982,19 +1955,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>302</v>
+      </c>
+      <c r="C1" t="s">
         <v>303</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>304</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>305</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>306</v>
-      </c>
-      <c r="F1" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -2002,135 +1975,135 @@
         <v>33</v>
       </c>
       <c r="B2" t="s">
+        <v>307</v>
+      </c>
+      <c r="C2" t="s">
         <v>308</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>309</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>310</v>
-      </c>
-      <c r="E2" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s">
+        <v>311</v>
+      </c>
+      <c r="C3" t="s">
         <v>312</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>313</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>314</v>
-      </c>
-      <c r="E3" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
+        <v>315</v>
+      </c>
+      <c r="C4" t="s">
         <v>316</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>317</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>318</v>
-      </c>
-      <c r="E4" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B5" t="s">
+        <v>319</v>
+      </c>
+      <c r="C5" t="s">
         <v>320</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>321</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>322</v>
-      </c>
-      <c r="E5" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6" t="s">
+        <v>323</v>
+      </c>
+      <c r="C6" t="s">
         <v>324</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>325</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>326</v>
-      </c>
-      <c r="E6" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B7" t="s">
+        <v>327</v>
+      </c>
+      <c r="C7" t="s">
         <v>328</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>329</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>330</v>
-      </c>
-      <c r="E7" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B8" t="s">
+        <v>319</v>
+      </c>
+      <c r="C8" t="s">
         <v>320</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>321</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>322</v>
-      </c>
-      <c r="E8" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B9" t="s">
+        <v>331</v>
+      </c>
+      <c r="C9" t="s">
         <v>332</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>333</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>334</v>
-      </c>
-      <c r="E9" t="s">
-        <v>335</v>
       </c>
     </row>
   </sheetData>
@@ -2149,22 +2122,22 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>335</v>
+      </c>
+      <c r="C1" t="s">
         <v>336</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>337</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>338</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>200</v>
+      </c>
+      <c r="G1" t="s">
         <v>339</v>
-      </c>
-      <c r="F1" t="s">
-        <v>201</v>
-      </c>
-      <c r="G1" t="s">
-        <v>340</v>
       </c>
     </row>
   </sheetData>
@@ -2183,19 +2156,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D1" t="s">
         <v>341</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
+        <v>200</v>
+      </c>
+      <c r="F1" t="s">
         <v>342</v>
-      </c>
-      <c r="E1" t="s">
-        <v>201</v>
-      </c>
-      <c r="F1" t="s">
-        <v>343</v>
       </c>
     </row>
   </sheetData>
@@ -2211,16 +2184,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B1" t="s">
+        <v>343</v>
+      </c>
+      <c r="C1" t="s">
         <v>344</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>345</v>
-      </c>
-      <c r="D1" t="s">
-        <v>346</v>
       </c>
     </row>
   </sheetData>
@@ -2236,16 +2209,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>346</v>
+      </c>
+      <c r="B1" t="s">
         <v>347</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>200</v>
+      </c>
+      <c r="D1" t="s">
         <v>348</v>
-      </c>
-      <c r="C1" t="s">
-        <v>201</v>
-      </c>
-      <c r="D1" t="s">
-        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -2264,34 +2237,34 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C1" t="s">
         <v>107</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>108</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>109</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>110</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>111</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>112</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>113</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>114</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>115</v>
-      </c>
-      <c r="K1" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -2299,180 +2272,180 @@
         <v>33</v>
       </c>
       <c r="B2" t="s">
+        <v>116</v>
+      </c>
+      <c r="G2" t="s">
         <v>117</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>118</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
+        <v>118</v>
+      </c>
+      <c r="K2" t="s">
         <v>119</v>
-      </c>
-      <c r="J2" t="s">
-        <v>119</v>
-      </c>
-      <c r="K2" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s">
+        <v>120</v>
+      </c>
+      <c r="G3" t="s">
         <v>121</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>122</v>
-      </c>
-      <c r="H3" t="s">
-        <v>123</v>
       </c>
       <c r="I3">
         <v>28</v>
       </c>
       <c r="J3" t="s">
+        <v>123</v>
+      </c>
+      <c r="K3" t="s">
         <v>124</v>
-      </c>
-      <c r="K3" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
+        <v>125</v>
+      </c>
+      <c r="G4" t="s">
         <v>126</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>127</v>
-      </c>
-      <c r="H4" t="s">
-        <v>128</v>
       </c>
       <c r="I4">
         <v>30</v>
       </c>
       <c r="J4" t="s">
+        <v>128</v>
+      </c>
+      <c r="K4" t="s">
         <v>129</v>
-      </c>
-      <c r="K4" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B5" t="s">
+        <v>130</v>
+      </c>
+      <c r="G5" t="s">
         <v>131</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>132</v>
-      </c>
-      <c r="H5" t="s">
-        <v>133</v>
       </c>
       <c r="I5">
         <v>35</v>
       </c>
       <c r="J5" t="s">
+        <v>133</v>
+      </c>
+      <c r="K5" t="s">
         <v>134</v>
-      </c>
-      <c r="K5" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6" t="s">
+        <v>135</v>
+      </c>
+      <c r="G6" t="s">
         <v>136</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>137</v>
-      </c>
-      <c r="H6" t="s">
-        <v>138</v>
       </c>
       <c r="I6">
         <v>30</v>
       </c>
       <c r="J6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B7" t="s">
+        <v>139</v>
+      </c>
+      <c r="G7" t="s">
         <v>140</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>141</v>
-      </c>
-      <c r="H7" t="s">
-        <v>142</v>
       </c>
       <c r="I7">
         <v>30</v>
       </c>
       <c r="J7" t="s">
+        <v>142</v>
+      </c>
+      <c r="K7" t="s">
         <v>143</v>
-      </c>
-      <c r="K7" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B8" t="s">
+        <v>144</v>
+      </c>
+      <c r="G8" t="s">
         <v>145</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>146</v>
-      </c>
-      <c r="H8" t="s">
-        <v>147</v>
       </c>
       <c r="I8">
         <v>30</v>
       </c>
       <c r="J8" t="s">
+        <v>147</v>
+      </c>
+      <c r="K8" t="s">
         <v>148</v>
-      </c>
-      <c r="K8" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G9" t="s">
+        <v>149</v>
+      </c>
+      <c r="H9" t="s">
         <v>150</v>
-      </c>
-      <c r="H9" t="s">
-        <v>151</v>
       </c>
       <c r="I9">
         <v>35</v>
       </c>
       <c r="J9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -2491,34 +2464,34 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C1" t="s">
         <v>153</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>154</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>155</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>156</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>157</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>158</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>159</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>160</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>161</v>
-      </c>
-      <c r="K1" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -2526,159 +2499,159 @@
         <v>33</v>
       </c>
       <c r="B2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C2" t="s">
         <v>163</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>164</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
+        <v>164</v>
+      </c>
+      <c r="G2" t="s">
         <v>165</v>
-      </c>
-      <c r="E2" t="s">
-        <v>165</v>
-      </c>
-      <c r="G2" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C3" t="s">
+        <v>163</v>
+      </c>
+      <c r="D3" t="s">
         <v>167</v>
       </c>
-      <c r="C3" t="s">
-        <v>164</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
+        <v>167</v>
+      </c>
+      <c r="G3" t="s">
         <v>168</v>
-      </c>
-      <c r="E3" t="s">
-        <v>168</v>
-      </c>
-      <c r="G3" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
+        <v>169</v>
+      </c>
+      <c r="C4" t="s">
+        <v>163</v>
+      </c>
+      <c r="D4" t="s">
         <v>170</v>
       </c>
-      <c r="C4" t="s">
-        <v>164</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
+        <v>170</v>
+      </c>
+      <c r="G4" t="s">
         <v>171</v>
-      </c>
-      <c r="E4" t="s">
-        <v>171</v>
-      </c>
-      <c r="G4" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B5" t="s">
+        <v>172</v>
+      </c>
+      <c r="C5" t="s">
+        <v>163</v>
+      </c>
+      <c r="D5" t="s">
         <v>173</v>
       </c>
-      <c r="C5" t="s">
-        <v>164</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
+        <v>173</v>
+      </c>
+      <c r="G5" t="s">
         <v>174</v>
-      </c>
-      <c r="E5" t="s">
-        <v>174</v>
-      </c>
-      <c r="G5" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6" t="s">
+        <v>175</v>
+      </c>
+      <c r="C6" t="s">
+        <v>163</v>
+      </c>
+      <c r="D6" t="s">
         <v>176</v>
       </c>
-      <c r="C6" t="s">
-        <v>164</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
+        <v>176</v>
+      </c>
+      <c r="G6" t="s">
         <v>177</v>
-      </c>
-      <c r="E6" t="s">
-        <v>177</v>
-      </c>
-      <c r="G6" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B7" t="s">
+        <v>178</v>
+      </c>
+      <c r="C7" t="s">
+        <v>163</v>
+      </c>
+      <c r="D7" t="s">
         <v>179</v>
       </c>
-      <c r="C7" t="s">
-        <v>164</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
+        <v>179</v>
+      </c>
+      <c r="G7" t="s">
         <v>180</v>
-      </c>
-      <c r="E7" t="s">
-        <v>180</v>
-      </c>
-      <c r="G7" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B8" t="s">
+        <v>181</v>
+      </c>
+      <c r="C8" t="s">
+        <v>163</v>
+      </c>
+      <c r="D8" t="s">
         <v>182</v>
       </c>
-      <c r="C8" t="s">
-        <v>164</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
+        <v>182</v>
+      </c>
+      <c r="G8" t="s">
         <v>183</v>
-      </c>
-      <c r="E8" t="s">
-        <v>183</v>
-      </c>
-      <c r="G8" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B9" t="s">
+        <v>184</v>
+      </c>
+      <c r="C9" t="s">
+        <v>163</v>
+      </c>
+      <c r="D9" t="s">
         <v>185</v>
       </c>
-      <c r="C9" t="s">
-        <v>164</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
+        <v>185</v>
+      </c>
+      <c r="G9" t="s">
         <v>186</v>
-      </c>
-      <c r="E9" t="s">
-        <v>186</v>
-      </c>
-      <c r="G9" t="s">
-        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -2697,46 +2670,46 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C1" t="s">
         <v>188</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>189</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>190</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>191</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>192</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>193</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>194</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>195</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>196</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>197</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>198</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>199</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>200</v>
-      </c>
-      <c r="O1" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -2744,10 +2717,10 @@
         <v>33</v>
       </c>
       <c r="B2" t="s">
+        <v>201</v>
+      </c>
+      <c r="E2" t="s">
         <v>202</v>
-      </c>
-      <c r="E2" t="s">
-        <v>203</v>
       </c>
       <c r="G2">
         <v>3923</v>
@@ -2762,7 +2735,7 @@
         <v>40014600</v>
       </c>
       <c r="O2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -2770,10 +2743,10 @@
         <v>33</v>
       </c>
       <c r="B3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E3" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="G3">
         <v>3959</v>
@@ -2788,7 +2761,7 @@
         <v>40381800</v>
       </c>
       <c r="O3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -2796,10 +2769,10 @@
         <v>33</v>
       </c>
       <c r="B4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="G4">
         <v>4894</v>
@@ -2814,7 +2787,7 @@
         <v>49918800</v>
       </c>
       <c r="O4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -2822,10 +2795,10 @@
         <v>33</v>
       </c>
       <c r="B5" t="s">
+        <v>206</v>
+      </c>
+      <c r="E5" t="s">
         <v>207</v>
-      </c>
-      <c r="E5" t="s">
-        <v>208</v>
       </c>
       <c r="G5">
         <v>4836</v>
@@ -2840,18 +2813,18 @@
         <v>49327200</v>
       </c>
       <c r="O5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
+        <v>208</v>
+      </c>
+      <c r="E6" t="s">
         <v>209</v>
-      </c>
-      <c r="E6" t="s">
-        <v>210</v>
       </c>
       <c r="G6">
         <v>660</v>
@@ -2866,18 +2839,18 @@
         <v>7920000</v>
       </c>
       <c r="O6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B7" t="s">
+        <v>210</v>
+      </c>
+      <c r="E7" t="s">
         <v>211</v>
-      </c>
-      <c r="E7" t="s">
-        <v>212</v>
       </c>
       <c r="G7">
         <v>1611</v>
@@ -2889,18 +2862,18 @@
         <v>19332000</v>
       </c>
       <c r="O7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B8" t="s">
+        <v>212</v>
+      </c>
+      <c r="E8" t="s">
         <v>213</v>
-      </c>
-      <c r="E8" t="s">
-        <v>214</v>
       </c>
       <c r="G8">
         <v>2333</v>
@@ -2912,18 +2885,18 @@
         <v>27996000</v>
       </c>
       <c r="O8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
+        <v>214</v>
+      </c>
+      <c r="E9" t="s">
         <v>215</v>
-      </c>
-      <c r="E9" t="s">
-        <v>216</v>
       </c>
       <c r="G9">
         <v>1242</v>
@@ -2935,18 +2908,18 @@
         <v>14904000</v>
       </c>
       <c r="O9" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E10" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G10">
         <v>1887</v>
@@ -2958,18 +2931,18 @@
         <v>22644000</v>
       </c>
       <c r="O10" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
+        <v>217</v>
+      </c>
+      <c r="E11" t="s">
         <v>218</v>
-      </c>
-      <c r="E11" t="s">
-        <v>219</v>
       </c>
       <c r="G11">
         <v>2191</v>
@@ -2981,18 +2954,18 @@
         <v>26292000</v>
       </c>
       <c r="O11" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B12" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E12" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G12">
         <v>715</v>
@@ -3004,18 +2977,18 @@
         <v>8409115</v>
       </c>
       <c r="O12" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E13" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G13">
         <v>1111</v>
@@ -3027,18 +3000,18 @@
         <v>13066471</v>
       </c>
       <c r="O13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B14" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E14" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G14">
         <v>1720</v>
@@ -3050,18 +3023,18 @@
         <v>20228920</v>
       </c>
       <c r="O14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E15" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G15">
         <v>1389</v>
@@ -3073,18 +3046,18 @@
         <v>13612200</v>
       </c>
       <c r="O15" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B16" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E16" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G16">
         <v>1063</v>
@@ -3096,18 +3069,18 @@
         <v>13074900</v>
       </c>
       <c r="O16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B17" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E17" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G17">
         <v>1510</v>
@@ -3119,18 +3092,18 @@
         <v>18573000</v>
       </c>
       <c r="O17" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B18" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E18" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G18">
         <v>753</v>
@@ -3142,18 +3115,18 @@
         <v>7906500</v>
       </c>
       <c r="O18" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B19" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E19" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G19">
         <v>1268</v>
@@ -3165,18 +3138,18 @@
         <v>13314000</v>
       </c>
       <c r="O19" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E20" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G20">
         <v>1733</v>
@@ -3188,18 +3161,18 @@
         <v>18196500</v>
       </c>
       <c r="O20" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B21" t="s">
+        <v>228</v>
+      </c>
+      <c r="E21" t="s">
         <v>229</v>
-      </c>
-      <c r="E21" t="s">
-        <v>230</v>
       </c>
       <c r="G21">
         <v>3336</v>
@@ -3211,18 +3184,18 @@
         <v>35028000</v>
       </c>
       <c r="O21" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B22" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E22" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G22">
         <v>734</v>
@@ -3234,18 +3207,18 @@
         <v>8441000</v>
       </c>
       <c r="O22" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B23" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E23" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G23">
         <v>1063</v>
@@ -3257,18 +3230,18 @@
         <v>12224500</v>
       </c>
       <c r="O23" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B24" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E24" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G24">
         <v>1510</v>
@@ -3280,18 +3253,18 @@
         <v>17365000</v>
       </c>
       <c r="O24" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B25" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E25" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G25">
         <v>2096</v>
@@ -3303,7 +3276,7 @@
         <v>24104000</v>
       </c>
       <c r="O25" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -3322,88 +3295,88 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>234</v>
+      </c>
+      <c r="C1" t="s">
         <v>235</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>236</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>237</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>238</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>239</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>240</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>241</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>242</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>243</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>244</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>245</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>246</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>247</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>248</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>249</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>250</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>251</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>252</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>253</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>254</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>255</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>256</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>257</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>258</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>259</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>260</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>261</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="2" spans="1:29" x14ac:dyDescent="0.25">
@@ -3420,15 +3393,15 @@
         <v>1</v>
       </c>
       <c r="G2" t="s">
+        <v>262</v>
+      </c>
+      <c r="AC2" t="s">
         <v>263</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3">
         <v>19</v>
@@ -3440,15 +3413,15 @@
         <v>8</v>
       </c>
       <c r="G3" t="s">
+        <v>264</v>
+      </c>
+      <c r="AC3" t="s">
         <v>265</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4">
         <v>10</v>
@@ -3460,15 +3433,15 @@
         <v>5</v>
       </c>
       <c r="G4" t="s">
+        <v>266</v>
+      </c>
+      <c r="AC4" t="s">
         <v>267</v>
-      </c>
-      <c r="AC4" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B5">
         <v>43</v>
@@ -3480,15 +3453,15 @@
         <v>10</v>
       </c>
       <c r="G5" t="s">
+        <v>268</v>
+      </c>
+      <c r="AC5" t="s">
         <v>269</v>
-      </c>
-      <c r="AC5" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6">
         <v>2</v>
@@ -3500,15 +3473,15 @@
         <v>8</v>
       </c>
       <c r="G6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AC6" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B7">
         <v>5</v>
@@ -3520,15 +3493,15 @@
         <v>8</v>
       </c>
       <c r="G7" t="s">
+        <v>271</v>
+      </c>
+      <c r="AC7" t="s">
         <v>272</v>
-      </c>
-      <c r="AC7" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -3540,15 +3513,15 @@
         <v>8</v>
       </c>
       <c r="G8" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="AC8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B9">
         <v>14</v>
@@ -3560,10 +3533,10 @@
         <v>8</v>
       </c>
       <c r="G9" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="AC9" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
   </sheetData>
@@ -3582,16 +3555,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>275</v>
+      </c>
+      <c r="C1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E1" t="s">
         <v>276</v>
-      </c>
-      <c r="C1" t="s">
-        <v>107</v>
-      </c>
-      <c r="D1" t="s">
-        <v>112</v>
-      </c>
-      <c r="E1" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -3599,111 +3572,111 @@
         <v>33</v>
       </c>
       <c r="B2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C2" t="s">
         <v>278</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>279</v>
-      </c>
-      <c r="E2" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s">
+        <v>277</v>
+      </c>
+      <c r="C3" t="s">
         <v>278</v>
       </c>
-      <c r="C3" t="s">
-        <v>279</v>
-      </c>
       <c r="E3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
+        <v>277</v>
+      </c>
+      <c r="C4" t="s">
         <v>278</v>
       </c>
-      <c r="C4" t="s">
-        <v>279</v>
-      </c>
       <c r="E4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B5" t="s">
+        <v>277</v>
+      </c>
+      <c r="C5" t="s">
         <v>278</v>
       </c>
-      <c r="C5" t="s">
-        <v>279</v>
-      </c>
       <c r="E5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6" t="s">
+        <v>277</v>
+      </c>
+      <c r="C6" t="s">
         <v>278</v>
       </c>
-      <c r="C6" t="s">
-        <v>279</v>
-      </c>
       <c r="E6" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B7" t="s">
+        <v>277</v>
+      </c>
+      <c r="C7" t="s">
         <v>278</v>
       </c>
-      <c r="C7" t="s">
-        <v>279</v>
-      </c>
       <c r="E7" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B8" t="s">
+        <v>277</v>
+      </c>
+      <c r="C8" t="s">
         <v>278</v>
       </c>
-      <c r="C8" t="s">
-        <v>279</v>
-      </c>
       <c r="E8" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B9" t="s">
+        <v>277</v>
+      </c>
+      <c r="C9" t="s">
         <v>278</v>
       </c>
-      <c r="C9" t="s">
-        <v>279</v>
-      </c>
       <c r="E9" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
   </sheetData>
@@ -3722,16 +3695,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D1" t="s">
+        <v>287</v>
+      </c>
+      <c r="E1" t="s">
         <v>288</v>
-      </c>
-      <c r="E1" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -3739,87 +3712,87 @@
         <v>33</v>
       </c>
       <c r="B2" t="s">
+        <v>289</v>
+      </c>
+      <c r="C2" t="s">
         <v>290</v>
-      </c>
-      <c r="C2" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B5" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C6" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B7" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C7" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B8" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C8" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B9" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
   </sheetData>
@@ -3838,16 +3811,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C1" t="s">
+        <v>298</v>
+      </c>
+      <c r="D1" t="s">
         <v>299</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>300</v>
-      </c>
-      <c r="E1" t="s">
-        <v>301</v>
       </c>
     </row>
   </sheetData>
@@ -3866,10 +3839,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C1" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
   </sheetData>

</xml_diff>